<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-13 00:09 UTC
</commit_message>
<xml_diff>
--- a/data/50001309 - ZITRON COLOMBIA BUGA BUENAVENTURA.xlsx
+++ b/data/50001309 - ZITRON COLOMBIA BUGA BUENAVENTURA.xlsx
@@ -1960,13 +1960,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46073.418435266205</v>
+        <v>46073.58510193287</v>
       </c>
       <c r="C4" s="5">
-        <v>46092.55588627315</v>
+        <v>46092.72255293981</v>
       </c>
       <c r="D4" s="5">
-        <v>46110.58383400463</v>
+        <v>46110.750500671296</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -2009,13 +2009,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="8">
-        <v>46073.41843560185</v>
+        <v>46073.585102268524</v>
       </c>
       <c r="C5" s="8">
-        <v>46092.55585400463</v>
+        <v>46092.7225206713</v>
       </c>
       <c r="D5" s="8">
-        <v>46133.71069020833</v>
+        <v>46133.877356875004</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>28</v>
@@ -2074,13 +2074,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46073.41843590278</v>
+        <v>46073.58510256944</v>
       </c>
       <c r="C6" s="5">
-        <v>46092.55585476852</v>
+        <v>46092.722521435186</v>
       </c>
       <c r="D6" s="5">
-        <v>46092.55588672454</v>
+        <v>46092.7225533912</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -2139,13 +2139,13 @@
         <v>38</v>
       </c>
       <c r="B7" s="8">
-        <v>46073.418436168984</v>
+        <v>46073.58510283565</v>
       </c>
       <c r="C7" s="8">
-        <v>46092.555855451385</v>
+        <v>46092.722522118056</v>
       </c>
       <c r="D7" s="8">
-        <v>46092.55588655092</v>
+        <v>46092.722553217594</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>39</v>
@@ -2204,13 +2204,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="5">
-        <v>46073.41843644676</v>
+        <v>46073.58510311342</v>
       </c>
       <c r="C8" s="5">
-        <v>46092.55585597223</v>
+        <v>46092.722522638884</v>
       </c>
       <c r="D8" s="5">
-        <v>46127.702947349535</v>
+        <v>46127.86961401621</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -2269,13 +2269,13 @@
         <v>43</v>
       </c>
       <c r="B9" s="8">
-        <v>46073.41843670139</v>
+        <v>46073.58510336805</v>
       </c>
       <c r="C9" s="8">
-        <v>46092.55585672453</v>
+        <v>46092.7225233912</v>
       </c>
       <c r="D9" s="8">
-        <v>46092.55588813657</v>
+        <v>46092.722554803244</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>44</v>
@@ -2334,13 +2334,13 @@
         <v>45</v>
       </c>
       <c r="B10" s="5">
-        <v>46073.41843773148</v>
+        <v>46073.58510439815</v>
       </c>
       <c r="C10" s="5">
-        <v>46107.617371458335</v>
+        <v>46107.784038125</v>
       </c>
       <c r="D10" s="5">
-        <v>46110.58391736111</v>
+        <v>46110.75058402777</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>46</v>
@@ -2383,13 +2383,13 @@
         <v>48</v>
       </c>
       <c r="B11" s="8">
-        <v>46073.418436238426</v>
+        <v>46073.5851029051</v>
       </c>
       <c r="C11" s="8">
-        <v>46097.37499174768</v>
+        <v>46097.54165841435</v>
       </c>
       <c r="D11" s="8">
-        <v>46097.375012986115</v>
+        <v>46097.54167965278</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>49</v>
@@ -2448,13 +2448,13 @@
         <v>51</v>
       </c>
       <c r="B12" s="5">
-        <v>46073.418437141205</v>
+        <v>46073.58510380787</v>
       </c>
       <c r="C12" s="5">
-        <v>46097.37504665509</v>
+        <v>46097.541713321756</v>
       </c>
       <c r="D12" s="5">
-        <v>46100.605553622685</v>
+        <v>46100.77222028935</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>52</v>
@@ -2513,13 +2513,13 @@
         <v>54</v>
       </c>
       <c r="B13" s="8">
-        <v>46073.41843752315</v>
+        <v>46073.58510418981</v>
       </c>
       <c r="C13" s="8">
-        <v>46097.37509494213</v>
+        <v>46097.541761608794</v>
       </c>
       <c r="D13" s="8">
-        <v>46097.37511282407</v>
+        <v>46097.54177949074</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>55</v>
@@ -2578,13 +2578,13 @@
         <v>57</v>
       </c>
       <c r="B14" s="5">
-        <v>46073.41843784723</v>
+        <v>46073.585104513884</v>
       </c>
       <c r="C14" s="5">
-        <v>46107.61735378472</v>
+        <v>46107.78402045139</v>
       </c>
       <c r="D14" s="5">
-        <v>46107.61737211805</v>
+        <v>46107.784038784725</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>58</v>
@@ -2643,13 +2643,13 @@
         <v>61</v>
       </c>
       <c r="B15" s="8">
-        <v>46073.41843815972</v>
+        <v>46073.58510482639</v>
       </c>
       <c r="C15" s="8">
-        <v>46107.61755152778</v>
+        <v>46107.78421819444</v>
       </c>
       <c r="D15" s="8">
-        <v>46110.58398484954</v>
+        <v>46110.7506515162</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>62</v>
@@ -2692,13 +2692,13 @@
         <v>64</v>
       </c>
       <c r="B16" s="5">
-        <v>46073.41843875</v>
+        <v>46073.58510541667</v>
       </c>
       <c r="C16" s="5">
-        <v>46097.37521457176</v>
+        <v>46097.54188123843</v>
       </c>
       <c r="D16" s="5">
-        <v>46097.37523175926</v>
+        <v>46097.54189842593</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>65</v>
@@ -2757,13 +2757,13 @@
         <v>67</v>
       </c>
       <c r="B17" s="8">
-        <v>46073.41843846065</v>
+        <v>46073.58510512731</v>
       </c>
       <c r="C17" s="8">
-        <v>46107.61750743055</v>
+        <v>46107.78417409722</v>
       </c>
       <c r="D17" s="8">
-        <v>46107.617520914355</v>
+        <v>46107.78418758102</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>68</v>
@@ -2822,13 +2822,13 @@
         <v>70</v>
       </c>
       <c r="B18" s="5">
-        <v>46073.418439375004</v>
+        <v>46073.58510604167</v>
       </c>
       <c r="C18" s="5">
-        <v>46097.37523667824</v>
+        <v>46097.54190334491</v>
       </c>
       <c r="D18" s="5">
-        <v>46100.6058175463</v>
+        <v>46100.77248421297</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>71</v>
@@ -2887,13 +2887,13 @@
         <v>74</v>
       </c>
       <c r="B19" s="8">
-        <v>46073.63271445602</v>
+        <v>46073.799381122684</v>
       </c>
       <c r="C19" s="8">
-        <v>46107.61753712963</v>
+        <v>46107.7842037963</v>
       </c>
       <c r="D19" s="8">
-        <v>46107.61755222222</v>
+        <v>46107.78421888889</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>75</v>
@@ -2952,13 +2952,13 @@
         <v>77</v>
       </c>
       <c r="B20" s="5">
-        <v>46073.4184365625</v>
+        <v>46073.58510322917</v>
       </c>
       <c r="C20" s="5">
-        <v>46097.37527456018</v>
+        <v>46097.54194122685</v>
       </c>
       <c r="D20" s="5">
-        <v>46100.6058733449</v>
+        <v>46100.772540011574</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>78</v>
@@ -3017,11 +3017,11 @@
         <v>82</v>
       </c>
       <c r="B21" s="8">
-        <v>46073.41843696759</v>
+        <v>46073.585103634265</v>
       </c>
       <c r="C21" s="9"/>
       <c r="D21" s="8">
-        <v>46174.4692159375</v>
+        <v>46174.63588260417</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>83</v>
@@ -3064,13 +3064,13 @@
         <v>85</v>
       </c>
       <c r="B22" s="5">
-        <v>46073.418437326385</v>
+        <v>46073.58510399306</v>
       </c>
       <c r="C22" s="5">
-        <v>46174.468762372686</v>
+        <v>46174.63542903935</v>
       </c>
       <c r="D22" s="5">
-        <v>46174.46876393519</v>
+        <v>46174.63543060185</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>86</v>
@@ -3129,13 +3129,13 @@
         <v>92</v>
       </c>
       <c r="B23" s="8">
-        <v>46073.41843763889</v>
+        <v>46073.58510430556</v>
       </c>
       <c r="C23" s="8">
-        <v>46114.358361122686</v>
+        <v>46114.52502778935</v>
       </c>
       <c r="D23" s="8">
-        <v>46169.66088693287</v>
+        <v>46169.827553599534</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>93</v>
@@ -3190,13 +3190,13 @@
         <v>95</v>
       </c>
       <c r="B24" s="5">
-        <v>46073.41843805555</v>
+        <v>46073.585104722224</v>
       </c>
       <c r="C24" s="5">
-        <v>46174.467621504635</v>
+        <v>46174.63428817129</v>
       </c>
       <c r="D24" s="5">
-        <v>46174.467623136574</v>
+        <v>46174.634289803245</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>96</v>
@@ -3251,13 +3251,13 @@
         <v>98</v>
       </c>
       <c r="B25" s="8">
-        <v>46073.41843921297</v>
+        <v>46073.585105879625</v>
       </c>
       <c r="C25" s="8">
-        <v>46174.46913729167</v>
+        <v>46174.63580395833</v>
       </c>
       <c r="D25" s="8">
-        <v>46174.469138622684</v>
+        <v>46174.63580528935</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>99</v>
@@ -3316,13 +3316,13 @@
         <v>101</v>
       </c>
       <c r="B26" s="5">
-        <v>46073.41843949074</v>
+        <v>46073.58510615741</v>
       </c>
       <c r="C26" s="5">
-        <v>46097.37537148148</v>
+        <v>46097.54203814815</v>
       </c>
       <c r="D26" s="5">
-        <v>46169.66094572916</v>
+        <v>46169.827612395835</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>102</v>
@@ -3377,13 +3377,13 @@
         <v>104</v>
       </c>
       <c r="B27" s="8">
-        <v>46073.41843600695</v>
+        <v>46073.58510267361</v>
       </c>
       <c r="C27" s="8">
-        <v>46174.46889752315</v>
+        <v>46174.63556418981</v>
       </c>
       <c r="D27" s="8">
-        <v>46174.46889885417</v>
+        <v>46174.63556552083</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>105</v>
@@ -3438,13 +3438,13 @@
         <v>107</v>
       </c>
       <c r="B28" s="5">
-        <v>46073.41843637732</v>
+        <v>46073.58510304398</v>
       </c>
       <c r="C28" s="5">
-        <v>46174.46920878472</v>
+        <v>46174.63587545139</v>
       </c>
       <c r="D28" s="5">
-        <v>46174.469210358795</v>
+        <v>46174.63587702546</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>108</v>
@@ -3503,13 +3503,13 @@
         <v>110</v>
       </c>
       <c r="B29" s="8">
-        <v>46073.41843672453</v>
+        <v>46073.585103391204</v>
       </c>
       <c r="C29" s="8">
-        <v>46097.37550635417</v>
+        <v>46097.54217302083</v>
       </c>
       <c r="D29" s="8">
-        <v>46169.66102943287</v>
+        <v>46169.827696099535</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>111</v>
@@ -3564,13 +3564,13 @@
         <v>113</v>
       </c>
       <c r="B30" s="5">
-        <v>46073.41843712963</v>
+        <v>46073.5851037963</v>
       </c>
       <c r="C30" s="5">
-        <v>46174.46908899306</v>
+        <v>46174.63575565972</v>
       </c>
       <c r="D30" s="5">
-        <v>46174.469090439816</v>
+        <v>46174.63575710648</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>114</v>
@@ -3625,13 +3625,13 @@
         <v>116</v>
       </c>
       <c r="B31" s="8">
-        <v>46073.41843752315</v>
+        <v>46073.58510418981</v>
       </c>
       <c r="C31" s="8">
-        <v>46114.35848997685</v>
+        <v>46114.52515664352</v>
       </c>
       <c r="D31" s="8">
-        <v>46169.661058645834</v>
+        <v>46169.8277253125</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>117</v>
@@ -3686,13 +3686,13 @@
         <v>119</v>
       </c>
       <c r="B32" s="5">
-        <v>46073.418437824075</v>
+        <v>46073.58510449074</v>
       </c>
       <c r="C32" s="5">
-        <v>46107.6196575463</v>
+        <v>46107.78632421297</v>
       </c>
       <c r="D32" s="5">
-        <v>46107.61967111111</v>
+        <v>46107.78633777778</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>120</v>
@@ -3751,13 +3751,13 @@
         <v>124</v>
       </c>
       <c r="B33" s="8">
-        <v>46073.418438125</v>
+        <v>46073.585104791666</v>
       </c>
       <c r="C33" s="8">
-        <v>46097.37578091436</v>
+        <v>46097.542447581014</v>
       </c>
       <c r="D33" s="8">
-        <v>46097.37578229167</v>
+        <v>46097.54244895834</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>125</v>
@@ -3812,13 +3812,13 @@
         <v>127</v>
       </c>
       <c r="B34" s="5">
-        <v>46073.41843854167</v>
+        <v>46073.58510520833</v>
       </c>
       <c r="C34" s="5">
-        <v>46107.619643576385</v>
+        <v>46107.78631024306</v>
       </c>
       <c r="D34" s="5">
-        <v>46107.61964510416</v>
+        <v>46107.78631177083</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>128</v>
@@ -3873,13 +3873,13 @@
         <v>130</v>
       </c>
       <c r="B35" s="8">
-        <v>46073.66294570602</v>
+        <v>46073.82961237269</v>
       </c>
       <c r="C35" s="8">
-        <v>46107.620129745366</v>
+        <v>46107.78679641204</v>
       </c>
       <c r="D35" s="8">
-        <v>46107.62016077546</v>
+        <v>46107.786827442134</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>131</v>
@@ -3938,13 +3938,13 @@
         <v>133</v>
       </c>
       <c r="B36" s="5">
-        <v>46077.477571944444</v>
+        <v>46077.644238611116</v>
       </c>
       <c r="C36" s="5">
-        <v>46107.62007344907</v>
+        <v>46107.78674011574</v>
       </c>
       <c r="D36" s="5">
-        <v>46107.62007592592</v>
+        <v>46107.786742592594</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>76</v>
@@ -4003,13 +4003,13 @@
         <v>135</v>
       </c>
       <c r="B37" s="8">
-        <v>46077.47910982639</v>
+        <v>46077.64577649305</v>
       </c>
       <c r="C37" s="8">
-        <v>46107.620115011574</v>
+        <v>46107.78678167824</v>
       </c>
       <c r="D37" s="8">
-        <v>46107.62011625</v>
+        <v>46107.786782916664</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>136</v>
@@ -4068,11 +4068,11 @@
         <v>138</v>
       </c>
       <c r="B38" s="5">
-        <v>46073.41843885416</v>
+        <v>46073.58510552083</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="5">
-        <v>46132.45700325232</v>
+        <v>46132.62366991898</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>139</v>
@@ -4117,13 +4117,13 @@
         <v>142</v>
       </c>
       <c r="B39" s="8">
-        <v>46073.41843910879</v>
+        <v>46073.58510577546</v>
       </c>
       <c r="C39" s="8">
-        <v>46098.35480232639</v>
+        <v>46098.52146899306</v>
       </c>
       <c r="D39" s="8">
-        <v>46169.66072833333</v>
+        <v>46169.827395</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>143</v>
@@ -4182,11 +4182,11 @@
         <v>147</v>
       </c>
       <c r="B40" s="5">
-        <v>46073.41843572917</v>
+        <v>46073.58510239584</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="5">
-        <v>46169.66076061343</v>
+        <v>46169.82742728009</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>148</v>
@@ -4245,11 +4245,11 @@
         <v>151</v>
       </c>
       <c r="B41" s="8">
-        <v>46090.74166175926</v>
+        <v>46090.908328425925</v>
       </c>
       <c r="C41" s="9"/>
       <c r="D41" s="8">
-        <v>46169.66081543981</v>
+        <v>46169.827482106484</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>150</v>
@@ -4306,11 +4306,11 @@
         <v>153</v>
       </c>
       <c r="B42" s="5">
-        <v>46090.74171902778</v>
+        <v>46090.90838569445</v>
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="5">
-        <v>46110.59346440972</v>
+        <v>46110.760131076386</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>154</v>
@@ -4369,11 +4369,11 @@
         <v>158</v>
       </c>
       <c r="B43" s="8">
-        <v>46109.732552511574</v>
+        <v>46109.899219178245</v>
       </c>
       <c r="C43" s="9"/>
       <c r="D43" s="8">
-        <v>46110.593077557874</v>
+        <v>46110.75974422454</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>159</v>
@@ -4422,11 +4422,11 @@
         <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46109.732567037034</v>
+        <v>46109.899233703705</v>
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="5">
-        <v>46110.59310758102</v>
+        <v>46110.75977424769</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>159</v>
@@ -4475,11 +4475,11 @@
         <v>162</v>
       </c>
       <c r="B45" s="8">
-        <v>46109.73257665509</v>
+        <v>46109.899243321765</v>
       </c>
       <c r="C45" s="9"/>
       <c r="D45" s="8">
-        <v>46110.59312627315</v>
+        <v>46110.75979293982</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>159</v>
@@ -4528,11 +4528,11 @@
         <v>163</v>
       </c>
       <c r="B46" s="5">
-        <v>46109.73258497685</v>
+        <v>46109.89925164352</v>
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="5">
-        <v>46110.59315353009</v>
+        <v>46110.75982019676</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>159</v>
@@ -4581,11 +4581,11 @@
         <v>164</v>
       </c>
       <c r="B47" s="8">
-        <v>46109.73259269676</v>
+        <v>46109.899259363425</v>
       </c>
       <c r="C47" s="9"/>
       <c r="D47" s="8">
-        <v>46110.59316923611</v>
+        <v>46110.759835902776</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>159</v>
@@ -4634,11 +4634,11 @@
         <v>165</v>
       </c>
       <c r="B48" s="5">
-        <v>46109.73259969907</v>
+        <v>46109.89926636574</v>
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="5">
-        <v>46110.59320403935</v>
+        <v>46110.75987070602</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>166</v>
@@ -4687,11 +4687,11 @@
         <v>167</v>
       </c>
       <c r="B49" s="8">
-        <v>46109.732606122685</v>
+        <v>46109.89927278935</v>
       </c>
       <c r="C49" s="9"/>
       <c r="D49" s="8">
-        <v>46110.593210300925</v>
+        <v>46110.7598769676</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>159</v>
@@ -4740,11 +4740,11 @@
         <v>168</v>
       </c>
       <c r="B50" s="5">
-        <v>46109.73261258102</v>
+        <v>46109.899279247686</v>
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="5">
-        <v>46110.59323506945</v>
+        <v>46110.759901736106</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>159</v>
@@ -4793,11 +4793,11 @@
         <v>169</v>
       </c>
       <c r="B51" s="8">
-        <v>46109.73261953704</v>
+        <v>46109.899286203705</v>
       </c>
       <c r="C51" s="9"/>
       <c r="D51" s="8">
-        <v>46110.59325601852</v>
+        <v>46110.75992268519</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>159</v>
@@ -4846,11 +4846,11 @@
         <v>170</v>
       </c>
       <c r="B52" s="5">
-        <v>46109.73262581018</v>
+        <v>46109.89929247685</v>
       </c>
       <c r="C52" s="6"/>
       <c r="D52" s="5">
-        <v>46110.59328408565</v>
+        <v>46110.75995075231</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>159</v>
@@ -4899,11 +4899,11 @@
         <v>171</v>
       </c>
       <c r="B53" s="8">
-        <v>46109.73263271991</v>
+        <v>46109.899299386576</v>
       </c>
       <c r="C53" s="9"/>
       <c r="D53" s="8">
-        <v>46110.59331172454</v>
+        <v>46110.7599783912</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>159</v>
@@ -4952,11 +4952,11 @@
         <v>172</v>
       </c>
       <c r="B54" s="5">
-        <v>46109.73263829861</v>
+        <v>46109.89930496528</v>
       </c>
       <c r="C54" s="6"/>
       <c r="D54" s="5">
-        <v>46110.59334957176</v>
+        <v>46110.760016238426</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>159</v>
@@ -5005,11 +5005,11 @@
         <v>173</v>
       </c>
       <c r="B55" s="8">
-        <v>46073.41843603009</v>
+        <v>46073.58510269676</v>
       </c>
       <c r="C55" s="9"/>
       <c r="D55" s="8">
-        <v>46083.483190810184</v>
+        <v>46083.64985747685</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>174</v>
@@ -5052,11 +5052,11 @@
         <v>176</v>
       </c>
       <c r="B56" s="5">
-        <v>46073.41843628472</v>
+        <v>46073.58510295139</v>
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46169.661230625</v>
+        <v>46169.82789729167</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>177</v>
@@ -5115,11 +5115,11 @@
         <v>181</v>
       </c>
       <c r="B57" s="8">
-        <v>46073.41843650463</v>
+        <v>46073.585103171295</v>
       </c>
       <c r="C57" s="9"/>
       <c r="D57" s="8">
-        <v>46099.982578634255</v>
+        <v>46100.14924530093</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>182</v>
@@ -5178,11 +5178,11 @@
         <v>186</v>
       </c>
       <c r="B58" s="5">
-        <v>46073.418436736116</v>
+        <v>46073.58510340277</v>
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46109.77036353009</v>
+        <v>46109.93703019676</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>187</v>
@@ -5225,11 +5225,11 @@
         <v>189</v>
       </c>
       <c r="B59" s="8">
-        <v>46073.418437037035</v>
+        <v>46073.58510370371</v>
       </c>
       <c r="C59" s="9"/>
       <c r="D59" s="8">
-        <v>46115.98568640046</v>
+        <v>46116.152353067126</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>190</v>
@@ -5288,11 +5288,11 @@
         <v>194</v>
       </c>
       <c r="B60" s="5">
-        <v>46073.41843726852</v>
+        <v>46073.585103935184</v>
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46120.08396771991</v>
+        <v>46120.250634386575</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>195</v>
@@ -5351,11 +5351,11 @@
         <v>198</v>
       </c>
       <c r="B61" s="8">
-        <v>46109.57515394676</v>
+        <v>46109.741820613424</v>
       </c>
       <c r="C61" s="9"/>
       <c r="D61" s="8">
-        <v>46120.00462409722</v>
+        <v>46120.17129076389</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>159</v>
@@ -5404,11 +5404,11 @@
         <v>201</v>
       </c>
       <c r="B62" s="5">
-        <v>46109.57517819444</v>
+        <v>46109.74184486111</v>
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="5">
-        <v>46120.00462581019</v>
+        <v>46120.17129247685</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>159</v>
@@ -5457,11 +5457,11 @@
         <v>202</v>
       </c>
       <c r="B63" s="8">
-        <v>46109.57518714121</v>
+        <v>46109.74185380787</v>
       </c>
       <c r="C63" s="9"/>
       <c r="D63" s="8">
-        <v>46120.00457158565</v>
+        <v>46120.17123825231</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>159</v>
@@ -5510,11 +5510,11 @@
         <v>203</v>
       </c>
       <c r="B64" s="5">
-        <v>46109.575196273145</v>
+        <v>46109.741862939816</v>
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46120.004573391205</v>
+        <v>46120.17124005787</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>159</v>
@@ -5563,11 +5563,11 @@
         <v>204</v>
       </c>
       <c r="B65" s="8">
-        <v>46109.57520357639</v>
+        <v>46109.74187024306</v>
       </c>
       <c r="C65" s="9"/>
       <c r="D65" s="8">
-        <v>46120.00457474537</v>
+        <v>46120.17124141204</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>159</v>
@@ -5616,11 +5616,11 @@
         <v>205</v>
       </c>
       <c r="B66" s="5">
-        <v>46109.57521052084</v>
+        <v>46109.7418771875</v>
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46120.00457619213</v>
+        <v>46120.17124285879</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>159</v>
@@ -5669,11 +5669,11 @@
         <v>206</v>
       </c>
       <c r="B67" s="8">
-        <v>46109.57521796296</v>
+        <v>46109.741884629635</v>
       </c>
       <c r="C67" s="9"/>
       <c r="D67" s="8">
-        <v>46120.004577604166</v>
+        <v>46120.17124427084</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>159</v>
@@ -5722,11 +5722,11 @@
         <v>207</v>
       </c>
       <c r="B68" s="5">
-        <v>46109.57522601852</v>
+        <v>46109.74189268518</v>
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46120.004579050925</v>
+        <v>46120.17124571759</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>159</v>
@@ -5775,11 +5775,11 @@
         <v>208</v>
       </c>
       <c r="B69" s="8">
-        <v>46109.575230937495</v>
+        <v>46109.741897604166</v>
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46120.004580451394</v>
+        <v>46120.17124711805</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>159</v>
@@ -5828,11 +5828,11 @@
         <v>209</v>
       </c>
       <c r="B70" s="5">
-        <v>46109.57523825231</v>
+        <v>46109.74190491898</v>
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46120.004582256945</v>
+        <v>46120.17124892361</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>159</v>
@@ -5881,11 +5881,11 @@
         <v>210</v>
       </c>
       <c r="B71" s="8">
-        <v>46109.5752435301</v>
+        <v>46109.74191019676</v>
       </c>
       <c r="C71" s="9"/>
       <c r="D71" s="8">
-        <v>46120.00458375</v>
+        <v>46120.171250416664</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>159</v>
@@ -5934,11 +5934,11 @@
         <v>211</v>
       </c>
       <c r="B72" s="5">
-        <v>46109.57714601852</v>
+        <v>46109.743812685185</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46120.004585312505</v>
+        <v>46120.17125197916</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>159</v>
@@ -5987,11 +5987,11 @@
         <v>212</v>
       </c>
       <c r="B73" s="8">
-        <v>46073.418437581015</v>
+        <v>46073.585104247686</v>
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="8">
-        <v>46122.00295383102</v>
+        <v>46122.16962049769</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>213</v>
@@ -6050,11 +6050,11 @@
         <v>215</v>
       </c>
       <c r="B74" s="5">
-        <v>46109.57618233796</v>
+        <v>46109.74284900463</v>
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46122.0062225</v>
+        <v>46122.17288916667</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>159</v>
@@ -6103,11 +6103,11 @@
         <v>218</v>
       </c>
       <c r="B75" s="8">
-        <v>46109.576195752314</v>
+        <v>46109.74286241898</v>
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="8">
-        <v>46122.0062241088</v>
+        <v>46122.17289077546</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>159</v>
@@ -6156,11 +6156,11 @@
         <v>219</v>
       </c>
       <c r="B76" s="5">
-        <v>46109.57620401621</v>
+        <v>46109.742870682865</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46122.00622606481</v>
+        <v>46122.17289273148</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>159</v>
@@ -6209,11 +6209,11 @@
         <v>220</v>
       </c>
       <c r="B77" s="8">
-        <v>46109.576210983796</v>
+        <v>46109.74287765047</v>
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46122.00622969907</v>
+        <v>46122.17289636574</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>159</v>
@@ -6262,11 +6262,11 @@
         <v>221</v>
       </c>
       <c r="B78" s="5">
-        <v>46109.576218194445</v>
+        <v>46109.742884861116</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46122.00623184028</v>
+        <v>46122.17289850695</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>159</v>
@@ -6315,11 +6315,11 @@
         <v>222</v>
       </c>
       <c r="B79" s="8">
-        <v>46109.57622412037</v>
+        <v>46109.742890787034</v>
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46122.0062331713</v>
+        <v>46122.17289983796</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>159</v>
@@ -6368,11 +6368,11 @@
         <v>223</v>
       </c>
       <c r="B80" s="5">
-        <v>46109.57622912037</v>
+        <v>46109.742895787036</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46122.00623462963</v>
+        <v>46122.1729012963</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>159</v>
@@ -6421,11 +6421,11 @@
         <v>224</v>
       </c>
       <c r="B81" s="8">
-        <v>46109.57623510416</v>
+        <v>46109.742901770835</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46122.0062359838</v>
+        <v>46122.17290265046</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>159</v>
@@ -6474,11 +6474,11 @@
         <v>225</v>
       </c>
       <c r="B82" s="5">
-        <v>46109.57624011574</v>
+        <v>46109.74290678241</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46122.00623732639</v>
+        <v>46122.17290399305</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>159</v>
@@ -6527,11 +6527,11 @@
         <v>226</v>
       </c>
       <c r="B83" s="8">
-        <v>46109.57624686343</v>
+        <v>46109.74291353009</v>
       </c>
       <c r="C83" s="9"/>
       <c r="D83" s="8">
-        <v>46122.006238773145</v>
+        <v>46122.17290543982</v>
       </c>
       <c r="E83" s="9" t="s">
         <v>159</v>
@@ -6580,11 +6580,11 @@
         <v>227</v>
       </c>
       <c r="B84" s="5">
-        <v>46109.57625226852</v>
+        <v>46109.74291893518</v>
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46122.006240104165</v>
+        <v>46122.17290677084</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>159</v>
@@ -6633,11 +6633,11 @@
         <v>228</v>
       </c>
       <c r="B85" s="8">
-        <v>46109.576505115736</v>
+        <v>46109.74317178241</v>
       </c>
       <c r="C85" s="9"/>
       <c r="D85" s="8">
-        <v>46122.00624185185</v>
+        <v>46122.17290851852</v>
       </c>
       <c r="E85" s="9" t="s">
         <v>159</v>
@@ -6686,11 +6686,11 @@
         <v>229</v>
       </c>
       <c r="B86" s="5">
-        <v>46073.418437824075</v>
+        <v>46073.58510449074</v>
       </c>
       <c r="C86" s="6"/>
       <c r="D86" s="5">
-        <v>46083.483383125</v>
+        <v>46083.65004979167</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>174</v>
@@ -6733,11 +6733,11 @@
         <v>231</v>
       </c>
       <c r="B87" s="8">
-        <v>46073.41843806713</v>
+        <v>46073.58510473379</v>
       </c>
       <c r="C87" s="9"/>
       <c r="D87" s="8">
-        <v>46174.46890556713</v>
+        <v>46174.6355722338</v>
       </c>
       <c r="E87" s="9" t="s">
         <v>232</v>
@@ -6796,11 +6796,11 @@
         <v>233</v>
       </c>
       <c r="B88" s="5">
-        <v>46073.41843615741</v>
+        <v>46073.58510282407</v>
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46174.46763211806</v>
+        <v>46174.634298784724</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>234</v>
@@ -6859,11 +6859,11 @@
         <v>236</v>
       </c>
       <c r="B89" s="8">
-        <v>46073.41843644676</v>
+        <v>46073.58510311342</v>
       </c>
       <c r="C89" s="9"/>
       <c r="D89" s="8">
-        <v>46184.08363760417</v>
+        <v>46184.250304270834</v>
       </c>
       <c r="E89" s="9" t="s">
         <v>237</v>
@@ -6922,13 +6922,13 @@
         <v>239</v>
       </c>
       <c r="B90" s="5">
-        <v>46073.66326402778</v>
+        <v>46073.82993069444</v>
       </c>
       <c r="C90" s="5">
-        <v>46109.57464366898</v>
+        <v>46109.74131033565</v>
       </c>
       <c r="D90" s="5">
-        <v>46111.34925854167</v>
+        <v>46111.51592520833</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>240</v>
@@ -6987,11 +6987,11 @@
         <v>242</v>
       </c>
       <c r="B91" s="8">
-        <v>46073.41843672453</v>
+        <v>46073.585103391204</v>
       </c>
       <c r="C91" s="9"/>
       <c r="D91" s="8">
-        <v>46109.82994694445</v>
+        <v>46109.99661361111</v>
       </c>
       <c r="E91" s="9" t="s">
         <v>243</v>
@@ -7034,11 +7034,11 @@
         <v>245</v>
       </c>
       <c r="B92" s="5">
-        <v>46073.41843708333</v>
+        <v>46073.585103749996</v>
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46142.00219809028</v>
+        <v>46142.16886475694</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>246</v>
@@ -7097,11 +7097,11 @@
         <v>247</v>
       </c>
       <c r="B93" s="8">
-        <v>46109.57807451389</v>
+        <v>46109.744741180555</v>
       </c>
       <c r="C93" s="9"/>
       <c r="D93" s="8">
-        <v>46142.003624467594</v>
+        <v>46142.17029113426</v>
       </c>
       <c r="E93" s="9" t="s">
         <v>159</v>
@@ -7150,11 +7150,11 @@
         <v>249</v>
       </c>
       <c r="B94" s="5">
-        <v>46109.578087870366</v>
+        <v>46109.74475453704</v>
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46142.00362599537</v>
+        <v>46142.170292662035</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>159</v>
@@ -7203,11 +7203,11 @@
         <v>250</v>
       </c>
       <c r="B95" s="8">
-        <v>46109.57809668982</v>
+        <v>46109.74476335648</v>
       </c>
       <c r="C95" s="9"/>
       <c r="D95" s="8">
-        <v>46142.00362715278</v>
+        <v>46142.17029381944</v>
       </c>
       <c r="E95" s="9" t="s">
         <v>159</v>
@@ -7256,11 +7256,11 @@
         <v>252</v>
       </c>
       <c r="B96" s="5">
-        <v>46109.57810452546</v>
+        <v>46109.74477119213</v>
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46142.00362855324</v>
+        <v>46142.17029521991</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>159</v>
@@ -7309,11 +7309,11 @@
         <v>253</v>
       </c>
       <c r="B97" s="8">
-        <v>46109.57811206019</v>
+        <v>46109.74477872685</v>
       </c>
       <c r="C97" s="9"/>
       <c r="D97" s="8">
-        <v>46142.00362988426</v>
+        <v>46142.170296550925</v>
       </c>
       <c r="E97" s="9" t="s">
         <v>159</v>
@@ -7362,11 +7362,11 @@
         <v>254</v>
       </c>
       <c r="B98" s="5">
-        <v>46109.57811986111</v>
+        <v>46109.74478652778</v>
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="5">
-        <v>46142.00363128472</v>
+        <v>46142.170297951394</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>159</v>
@@ -7415,11 +7415,11 @@
         <v>255</v>
       </c>
       <c r="B99" s="8">
-        <v>46109.578125740736</v>
+        <v>46109.74479240741</v>
       </c>
       <c r="C99" s="9"/>
       <c r="D99" s="8">
-        <v>46142.00363262731</v>
+        <v>46142.17029929398</v>
       </c>
       <c r="E99" s="9" t="s">
         <v>159</v>
@@ -7468,11 +7468,11 @@
         <v>256</v>
       </c>
       <c r="B100" s="5">
-        <v>46109.57813188658</v>
+        <v>46109.74479855324</v>
       </c>
       <c r="C100" s="6"/>
       <c r="D100" s="5">
-        <v>46142.00363388889</v>
+        <v>46142.17030055556</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>159</v>
@@ -7521,11 +7521,11 @@
         <v>257</v>
       </c>
       <c r="B101" s="8">
-        <v>46109.57813711806</v>
+        <v>46109.74480378472</v>
       </c>
       <c r="C101" s="9"/>
       <c r="D101" s="8">
-        <v>46142.00363528935</v>
+        <v>46142.17030195602</v>
       </c>
       <c r="E101" s="9" t="s">
         <v>159</v>
@@ -7574,11 +7574,11 @@
         <v>258</v>
       </c>
       <c r="B102" s="5">
-        <v>46109.57814349537</v>
+        <v>46109.74481016204</v>
       </c>
       <c r="C102" s="6"/>
       <c r="D102" s="5">
-        <v>46142.003636863425</v>
+        <v>46142.17030353009</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>159</v>
@@ -7627,11 +7627,11 @@
         <v>259</v>
       </c>
       <c r="B103" s="8">
-        <v>46109.578148773144</v>
+        <v>46109.744815439815</v>
       </c>
       <c r="C103" s="9"/>
       <c r="D103" s="8">
-        <v>46142.003614236106</v>
+        <v>46142.17028090278</v>
       </c>
       <c r="E103" s="9" t="s">
         <v>159</v>
@@ -7680,11 +7680,11 @@
         <v>260</v>
       </c>
       <c r="B104" s="5">
-        <v>46109.578153993054</v>
+        <v>46109.74482065972</v>
       </c>
       <c r="C104" s="6"/>
       <c r="D104" s="5">
-        <v>46142.003615821755</v>
+        <v>46142.17028248843</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>159</v>
@@ -7733,11 +7733,11 @@
         <v>261</v>
       </c>
       <c r="B105" s="8">
-        <v>46079.37245340278</v>
+        <v>46079.53912006944</v>
       </c>
       <c r="C105" s="9"/>
       <c r="D105" s="8">
-        <v>46160.00148028936</v>
+        <v>46160.16814695601</v>
       </c>
       <c r="E105" s="9" t="s">
         <v>262</v>
@@ -7796,11 +7796,11 @@
         <v>263</v>
       </c>
       <c r="B106" s="5">
-        <v>46109.578735034724</v>
+        <v>46109.74540170139</v>
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="5">
-        <v>46160.00207862268</v>
+        <v>46160.16874528935</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>159</v>
@@ -7849,11 +7849,11 @@
         <v>266</v>
       </c>
       <c r="B107" s="8">
-        <v>46109.57875049769</v>
+        <v>46109.74541716435</v>
       </c>
       <c r="C107" s="9"/>
       <c r="D107" s="8">
-        <v>46160.00208017361</v>
+        <v>46160.16874684028</v>
       </c>
       <c r="E107" s="9" t="s">
         <v>159</v>
@@ -7902,11 +7902,11 @@
         <v>269</v>
       </c>
       <c r="B108" s="5">
-        <v>46109.57875881944</v>
+        <v>46109.74542548611</v>
       </c>
       <c r="C108" s="6"/>
       <c r="D108" s="5">
-        <v>46160.002081388884</v>
+        <v>46160.168748055556</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>159</v>
@@ -7955,11 +7955,11 @@
         <v>271</v>
       </c>
       <c r="B109" s="8">
-        <v>46109.578765451384</v>
+        <v>46109.745432118056</v>
       </c>
       <c r="C109" s="9"/>
       <c r="D109" s="8">
-        <v>46160.00208288194</v>
+        <v>46160.16874954861</v>
       </c>
       <c r="E109" s="9" t="s">
         <v>159</v>
@@ -8008,11 +8008,11 @@
         <v>273</v>
       </c>
       <c r="B110" s="5">
-        <v>46109.57877140046</v>
+        <v>46109.745438067126</v>
       </c>
       <c r="C110" s="6"/>
       <c r="D110" s="5">
-        <v>46160.00208435185</v>
+        <v>46160.168751018515</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>159</v>
@@ -8061,11 +8061,11 @@
         <v>274</v>
       </c>
       <c r="B111" s="8">
-        <v>46109.57877733796</v>
+        <v>46109.74544400463</v>
       </c>
       <c r="C111" s="9"/>
       <c r="D111" s="8">
-        <v>46160.002086064815</v>
+        <v>46160.16875273148</v>
       </c>
       <c r="E111" s="9" t="s">
         <v>159</v>
@@ -8114,11 +8114,11 @@
         <v>275</v>
       </c>
       <c r="B112" s="5">
-        <v>46109.57878372685</v>
+        <v>46109.745450393515</v>
       </c>
       <c r="C112" s="6"/>
       <c r="D112" s="5">
-        <v>46160.00208740741</v>
+        <v>46160.168754074075</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>159</v>
@@ -8167,11 +8167,11 @@
         <v>276</v>
       </c>
       <c r="B113" s="8">
-        <v>46109.57878938658</v>
+        <v>46109.74545605324</v>
       </c>
       <c r="C113" s="9"/>
       <c r="D113" s="8">
-        <v>46160.00208873843</v>
+        <v>46160.16875540509</v>
       </c>
       <c r="E113" s="9" t="s">
         <v>159</v>
@@ -8220,11 +8220,11 @@
         <v>277</v>
       </c>
       <c r="B114" s="5">
-        <v>46109.578795208334</v>
+        <v>46109.745461875005</v>
       </c>
       <c r="C114" s="6"/>
       <c r="D114" s="5">
-        <v>46160.0020900463</v>
+        <v>46160.16875671296</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>159</v>
@@ -8273,11 +8273,11 @@
         <v>278</v>
       </c>
       <c r="B115" s="8">
-        <v>46109.57880268518</v>
+        <v>46109.74546935185</v>
       </c>
       <c r="C115" s="9"/>
       <c r="D115" s="8">
-        <v>46160.00209165509</v>
+        <v>46160.16875832176</v>
       </c>
       <c r="E115" s="9" t="s">
         <v>159</v>
@@ -8326,11 +8326,11 @@
         <v>279</v>
       </c>
       <c r="B116" s="5">
-        <v>46109.57881032408</v>
+        <v>46109.74547699074</v>
       </c>
       <c r="C116" s="6"/>
       <c r="D116" s="5">
-        <v>46160.00209300926</v>
+        <v>46160.16875967593</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>159</v>
@@ -8379,11 +8379,11 @@
         <v>280</v>
       </c>
       <c r="B117" s="8">
-        <v>46109.72923745371</v>
+        <v>46109.89590412037</v>
       </c>
       <c r="C117" s="9"/>
       <c r="D117" s="8">
-        <v>46160.002094375</v>
+        <v>46160.16876104167</v>
       </c>
       <c r="E117" s="9" t="s">
         <v>159</v>
@@ -8432,11 +8432,11 @@
         <v>281</v>
       </c>
       <c r="B118" s="5">
-        <v>46073.41843784723</v>
+        <v>46073.585104513884</v>
       </c>
       <c r="C118" s="6"/>
       <c r="D118" s="5">
-        <v>46162.001228946756</v>
+        <v>46162.16789561343</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>282</v>
@@ -8495,11 +8495,11 @@
         <v>284</v>
       </c>
       <c r="B119" s="8">
-        <v>46109.57846130787</v>
+        <v>46109.74512797454</v>
       </c>
       <c r="C119" s="9"/>
       <c r="D119" s="8">
-        <v>46162.00190447917</v>
+        <v>46162.168571145834</v>
       </c>
       <c r="E119" s="9" t="s">
         <v>159</v>
@@ -8548,11 +8548,11 @@
         <v>287</v>
       </c>
       <c r="B120" s="5">
-        <v>46109.578474594906</v>
+        <v>46109.74514126158</v>
       </c>
       <c r="C120" s="6"/>
       <c r="D120" s="5">
-        <v>46162.001906006946</v>
+        <v>46162.16857267361</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>288</v>
@@ -8601,11 +8601,11 @@
         <v>289</v>
       </c>
       <c r="B121" s="8">
-        <v>46109.57848200231</v>
+        <v>46109.74514866898</v>
       </c>
       <c r="C121" s="9"/>
       <c r="D121" s="8">
-        <v>46162.00190729166</v>
+        <v>46162.16857395833</v>
       </c>
       <c r="E121" s="9" t="s">
         <v>159</v>
@@ -8654,11 +8654,11 @@
         <v>290</v>
       </c>
       <c r="B122" s="5">
-        <v>46109.578489629625</v>
+        <v>46109.745156296296</v>
       </c>
       <c r="C122" s="6"/>
       <c r="D122" s="5">
-        <v>46162.00190856482</v>
+        <v>46162.16857523148</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>159</v>
@@ -8707,11 +8707,11 @@
         <v>291</v>
       </c>
       <c r="B123" s="8">
-        <v>46109.578497291666</v>
+        <v>46109.74516395833</v>
       </c>
       <c r="C123" s="9"/>
       <c r="D123" s="8">
-        <v>46162.00190974537</v>
+        <v>46162.168576412034</v>
       </c>
       <c r="E123" s="9" t="s">
         <v>159</v>
@@ -8760,11 +8760,11 @@
         <v>293</v>
       </c>
       <c r="B124" s="5">
-        <v>46109.578505219906</v>
+        <v>46109.74517188658</v>
       </c>
       <c r="C124" s="6"/>
       <c r="D124" s="5">
-        <v>46162.00191091435</v>
+        <v>46162.16857758102</v>
       </c>
       <c r="E124" s="6" t="s">
         <v>159</v>
@@ -8813,11 +8813,11 @@
         <v>294</v>
       </c>
       <c r="B125" s="8">
-        <v>46109.57851064815</v>
+        <v>46109.74517731481</v>
       </c>
       <c r="C125" s="9"/>
       <c r="D125" s="8">
-        <v>46162.001912164356</v>
+        <v>46162.16857883101</v>
       </c>
       <c r="E125" s="9" t="s">
         <v>159</v>
@@ -8866,11 +8866,11 @@
         <v>295</v>
       </c>
       <c r="B126" s="5">
-        <v>46109.57851770833</v>
+        <v>46109.745184375</v>
       </c>
       <c r="C126" s="6"/>
       <c r="D126" s="5">
-        <v>46162.00191356482</v>
+        <v>46162.16858023148</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>159</v>
@@ -8919,11 +8919,11 @@
         <v>296</v>
       </c>
       <c r="B127" s="8">
-        <v>46109.57852252315</v>
+        <v>46109.745189189816</v>
       </c>
       <c r="C127" s="9"/>
       <c r="D127" s="8">
-        <v>46162.001914837965</v>
+        <v>46162.16858150463</v>
       </c>
       <c r="E127" s="9" t="s">
         <v>159</v>
@@ -8972,11 +8972,11 @@
         <v>297</v>
       </c>
       <c r="B128" s="5">
-        <v>46109.57852923611</v>
+        <v>46109.74519590278</v>
       </c>
       <c r="C128" s="6"/>
       <c r="D128" s="5">
-        <v>46162.00191603009</v>
+        <v>46162.16858269676</v>
       </c>
       <c r="E128" s="6" t="s">
         <v>159</v>
@@ -9025,11 +9025,11 @@
         <v>298</v>
       </c>
       <c r="B129" s="8">
-        <v>46109.57853621528</v>
+        <v>46109.745202881946</v>
       </c>
       <c r="C129" s="9"/>
       <c r="D129" s="8">
-        <v>46162.00191730324</v>
+        <v>46162.168583969906</v>
       </c>
       <c r="E129" s="9" t="s">
         <v>159</v>
@@ -9078,11 +9078,11 @@
         <v>299</v>
       </c>
       <c r="B130" s="5">
-        <v>46109.57854275463</v>
+        <v>46109.74520942129</v>
       </c>
       <c r="C130" s="6"/>
       <c r="D130" s="5">
-        <v>46162.00191869213</v>
+        <v>46162.1685853588</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>159</v>
@@ -9131,11 +9131,11 @@
         <v>300</v>
       </c>
       <c r="B131" s="8">
-        <v>46073.41843810186</v>
+        <v>46073.585104768514</v>
       </c>
       <c r="C131" s="9"/>
       <c r="D131" s="8">
-        <v>46168.00112981482</v>
+        <v>46168.16779648148</v>
       </c>
       <c r="E131" s="9" t="s">
         <v>301</v>
@@ -9194,11 +9194,11 @@
         <v>302</v>
       </c>
       <c r="B132" s="5">
-        <v>46109.57860649306</v>
+        <v>46109.74527315972</v>
       </c>
       <c r="C132" s="6"/>
       <c r="D132" s="5">
-        <v>46168.00171320602</v>
+        <v>46168.16837987269</v>
       </c>
       <c r="E132" s="6" t="s">
         <v>159</v>
@@ -9247,11 +9247,11 @@
         <v>304</v>
       </c>
       <c r="B133" s="8">
-        <v>46109.57861914352</v>
+        <v>46109.74528581019</v>
       </c>
       <c r="C133" s="9"/>
       <c r="D133" s="8">
-        <v>46168.00171490741</v>
+        <v>46168.16838157407</v>
       </c>
       <c r="E133" s="9" t="s">
         <v>159</v>
@@ -9300,11 +9300,11 @@
         <v>305</v>
       </c>
       <c r="B134" s="5">
-        <v>46109.578627002316</v>
+        <v>46109.74529366898</v>
       </c>
       <c r="C134" s="6"/>
       <c r="D134" s="5">
-        <v>46168.001716087965</v>
+        <v>46168.16838275463</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>159</v>
@@ -9353,11 +9353,11 @@
         <v>306</v>
       </c>
       <c r="B135" s="8">
-        <v>46109.57863427083</v>
+        <v>46109.7453009375</v>
       </c>
       <c r="C135" s="9"/>
       <c r="D135" s="8">
-        <v>46168.0017172338</v>
+        <v>46168.16838390046</v>
       </c>
       <c r="E135" s="9" t="s">
         <v>159</v>
@@ -9406,11 +9406,11 @@
         <v>307</v>
       </c>
       <c r="B136" s="5">
-        <v>46109.57864179398</v>
+        <v>46109.74530846065</v>
       </c>
       <c r="C136" s="6"/>
       <c r="D136" s="5">
-        <v>46168.0017184375</v>
+        <v>46168.16838510417</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>159</v>
@@ -9459,11 +9459,11 @@
         <v>308</v>
       </c>
       <c r="B137" s="8">
-        <v>46109.578649097224</v>
+        <v>46109.74531576389</v>
       </c>
       <c r="C137" s="9"/>
       <c r="D137" s="8">
-        <v>46168.00171965278</v>
+        <v>46168.16838631945</v>
       </c>
       <c r="E137" s="9" t="s">
         <v>159</v>
@@ -9512,11 +9512,11 @@
         <v>309</v>
       </c>
       <c r="B138" s="5">
-        <v>46109.57865524305</v>
+        <v>46109.74532190972</v>
       </c>
       <c r="C138" s="6"/>
       <c r="D138" s="5">
-        <v>46168.001720949076</v>
+        <v>46168.16838761574</v>
       </c>
       <c r="E138" s="6" t="s">
         <v>159</v>
@@ -9565,11 +9565,11 @@
         <v>310</v>
       </c>
       <c r="B139" s="8">
-        <v>46109.57866271991</v>
+        <v>46109.74532938657</v>
       </c>
       <c r="C139" s="9"/>
       <c r="D139" s="8">
-        <v>46168.001722245375</v>
+        <v>46168.16838891203</v>
       </c>
       <c r="E139" s="9" t="s">
         <v>159</v>
@@ -9618,11 +9618,11 @@
         <v>311</v>
       </c>
       <c r="B140" s="5">
-        <v>46109.57866824074</v>
+        <v>46109.745334907406</v>
       </c>
       <c r="C140" s="6"/>
       <c r="D140" s="5">
-        <v>46168.00172342593</v>
+        <v>46168.16839009259</v>
       </c>
       <c r="E140" s="6" t="s">
         <v>159</v>
@@ -9671,11 +9671,11 @@
         <v>312</v>
       </c>
       <c r="B141" s="8">
-        <v>46109.578675324075</v>
+        <v>46109.74534199074</v>
       </c>
       <c r="C141" s="9"/>
       <c r="D141" s="8">
-        <v>46168.00172461805</v>
+        <v>46168.16839128472</v>
       </c>
       <c r="E141" s="9" t="s">
         <v>159</v>
@@ -9724,11 +9724,11 @@
         <v>313</v>
       </c>
       <c r="B142" s="5">
-        <v>46109.5786805324</v>
+        <v>46109.745347199074</v>
       </c>
       <c r="C142" s="6"/>
       <c r="D142" s="5">
-        <v>46168.00172576389</v>
+        <v>46168.168392430554</v>
       </c>
       <c r="E142" s="6" t="s">
         <v>159</v>
@@ -9777,11 +9777,11 @@
         <v>314</v>
       </c>
       <c r="B143" s="8">
-        <v>46109.57868723379</v>
+        <v>46109.745353900464</v>
       </c>
       <c r="C143" s="9"/>
       <c r="D143" s="8">
-        <v>46168.00172696759</v>
+        <v>46168.16839363426</v>
       </c>
       <c r="E143" s="9" t="s">
         <v>159</v>
@@ -9830,11 +9830,11 @@
         <v>315</v>
       </c>
       <c r="B144" s="5">
-        <v>46073.418437569446</v>
+        <v>46073.58510423611</v>
       </c>
       <c r="C144" s="6"/>
       <c r="D144" s="5">
-        <v>46110.58633215278</v>
+        <v>46110.752998819444</v>
       </c>
       <c r="E144" s="6" t="s">
         <v>316</v>
@@ -9893,11 +9893,11 @@
         <v>317</v>
       </c>
       <c r="B145" s="8">
-        <v>46109.57830168981</v>
+        <v>46109.74496835648</v>
       </c>
       <c r="C145" s="9"/>
       <c r="D145" s="8">
-        <v>46110.585254398145</v>
+        <v>46110.75192106482</v>
       </c>
       <c r="E145" s="9" t="s">
         <v>159</v>
@@ -9946,11 +9946,11 @@
         <v>319</v>
       </c>
       <c r="B146" s="5">
-        <v>46109.5783168287</v>
+        <v>46109.74498349537</v>
       </c>
       <c r="C146" s="6"/>
       <c r="D146" s="5">
-        <v>46110.58532917824</v>
+        <v>46110.75199584491</v>
       </c>
       <c r="E146" s="6" t="s">
         <v>159</v>
@@ -9999,11 +9999,11 @@
         <v>321</v>
       </c>
       <c r="B147" s="8">
-        <v>46109.57832538194</v>
+        <v>46109.74499204861</v>
       </c>
       <c r="C147" s="9"/>
       <c r="D147" s="8">
-        <v>46110.58536041666</v>
+        <v>46110.752027083334</v>
       </c>
       <c r="E147" s="9" t="s">
         <v>159</v>
@@ -10052,11 +10052,11 @@
         <v>323</v>
       </c>
       <c r="B148" s="5">
-        <v>46109.57833488426</v>
+        <v>46109.745001550924</v>
       </c>
       <c r="C148" s="6"/>
       <c r="D148" s="5">
-        <v>46110.58538596064</v>
+        <v>46110.752052627315</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>159</v>
@@ -10105,11 +10105,11 @@
         <v>324</v>
       </c>
       <c r="B149" s="8">
-        <v>46109.57834269676</v>
+        <v>46109.745009363425</v>
       </c>
       <c r="C149" s="9"/>
       <c r="D149" s="8">
-        <v>46110.58541353009</v>
+        <v>46110.75208019676</v>
       </c>
       <c r="E149" s="9" t="s">
         <v>159</v>
@@ -10158,11 +10158,11 @@
         <v>325</v>
       </c>
       <c r="B150" s="5">
-        <v>46109.5783517824</v>
+        <v>46109.74501844907</v>
       </c>
       <c r="C150" s="6"/>
       <c r="D150" s="5">
-        <v>46110.585444791664</v>
+        <v>46110.752111458336</v>
       </c>
       <c r="E150" s="6" t="s">
         <v>159</v>
@@ -10211,11 +10211,11 @@
         <v>327</v>
       </c>
       <c r="B151" s="8">
-        <v>46109.57835979167</v>
+        <v>46109.74502645833</v>
       </c>
       <c r="C151" s="9"/>
       <c r="D151" s="8">
-        <v>46110.58546973379</v>
+        <v>46110.752136400464</v>
       </c>
       <c r="E151" s="9" t="s">
         <v>159</v>
@@ -10264,11 +10264,11 @@
         <v>328</v>
       </c>
       <c r="B152" s="5">
-        <v>46109.57836712963</v>
+        <v>46109.745033796295</v>
       </c>
       <c r="C152" s="6"/>
       <c r="D152" s="5">
-        <v>46110.58549211806</v>
+        <v>46110.75215878472</v>
       </c>
       <c r="E152" s="6" t="s">
         <v>159</v>
@@ -10317,11 +10317,11 @@
         <v>330</v>
       </c>
       <c r="B153" s="8">
-        <v>46109.57837403935</v>
+        <v>46109.74504070602</v>
       </c>
       <c r="C153" s="9"/>
       <c r="D153" s="8">
-        <v>46110.58551409723</v>
+        <v>46110.752180763884</v>
       </c>
       <c r="E153" s="9" t="s">
         <v>159</v>
@@ -10370,11 +10370,11 @@
         <v>331</v>
       </c>
       <c r="B154" s="5">
-        <v>46109.57838075231</v>
+        <v>46109.74504741898</v>
       </c>
       <c r="C154" s="6"/>
       <c r="D154" s="5">
-        <v>46110.585538576386</v>
+        <v>46110.75220524306</v>
       </c>
       <c r="E154" s="6" t="s">
         <v>159</v>
@@ -10423,11 +10423,11 @@
         <v>332</v>
       </c>
       <c r="B155" s="8">
-        <v>46109.578389166665</v>
+        <v>46109.74505583334</v>
       </c>
       <c r="C155" s="9"/>
       <c r="D155" s="8">
-        <v>46110.5855633912</v>
+        <v>46110.75223005787</v>
       </c>
       <c r="E155" s="9" t="s">
         <v>159</v>
@@ -10476,11 +10476,11 @@
         <v>333</v>
       </c>
       <c r="B156" s="5">
-        <v>46109.57839761574</v>
+        <v>46109.74506428241</v>
       </c>
       <c r="C156" s="6"/>
       <c r="D156" s="5">
-        <v>46110.58560384259</v>
+        <v>46110.752270509256</v>
       </c>
       <c r="E156" s="6" t="s">
         <v>159</v>
@@ -10529,11 +10529,11 @@
         <v>335</v>
       </c>
       <c r="B157" s="8">
-        <v>46073.41843837963</v>
+        <v>46073.585105046295</v>
       </c>
       <c r="C157" s="9"/>
       <c r="D157" s="8">
-        <v>46110.588973715276</v>
+        <v>46110.75564038195</v>
       </c>
       <c r="E157" s="9" t="s">
         <v>336</v>
@@ -10592,11 +10592,11 @@
         <v>337</v>
       </c>
       <c r="B158" s="5">
-        <v>46109.578872812504</v>
+        <v>46109.74553947916</v>
       </c>
       <c r="C158" s="6"/>
       <c r="D158" s="5">
-        <v>46110.58816075232</v>
+        <v>46110.75482741898</v>
       </c>
       <c r="E158" s="6" t="s">
         <v>159</v>
@@ -10645,11 +10645,11 @@
         <v>339</v>
       </c>
       <c r="B159" s="8">
-        <v>46109.57888017361</v>
+        <v>46109.74554684028</v>
       </c>
       <c r="C159" s="9"/>
       <c r="D159" s="8">
-        <v>46110.58818361111</v>
+        <v>46110.75485027778</v>
       </c>
       <c r="E159" s="9" t="s">
         <v>159</v>
@@ -10698,11 +10698,11 @@
         <v>340</v>
       </c>
       <c r="B160" s="5">
-        <v>46109.57888747685</v>
+        <v>46109.74555414352</v>
       </c>
       <c r="C160" s="6"/>
       <c r="D160" s="5">
-        <v>46110.58820783565</v>
+        <v>46110.754874502316</v>
       </c>
       <c r="E160" s="6" t="s">
         <v>159</v>
@@ -10751,11 +10751,11 @@
         <v>341</v>
       </c>
       <c r="B161" s="8">
-        <v>46109.57889495371</v>
+        <v>46109.745561620366</v>
       </c>
       <c r="C161" s="9"/>
       <c r="D161" s="8">
-        <v>46110.58821543981</v>
+        <v>46110.754882106485</v>
       </c>
       <c r="E161" s="9" t="s">
         <v>159</v>
@@ -10804,11 +10804,11 @@
         <v>342</v>
       </c>
       <c r="B162" s="5">
-        <v>46109.57991605324</v>
+        <v>46109.746582719905</v>
       </c>
       <c r="C162" s="6"/>
       <c r="D162" s="5">
-        <v>46110.59171199074</v>
+        <v>46110.75837865741</v>
       </c>
       <c r="E162" s="6" t="s">
         <v>159</v>
@@ -10857,11 +10857,11 @@
         <v>343</v>
       </c>
       <c r="B163" s="8">
-        <v>46109.579953113425</v>
+        <v>46109.7466197801</v>
       </c>
       <c r="C163" s="9"/>
       <c r="D163" s="8">
-        <v>46110.58829914352</v>
+        <v>46110.754965810185</v>
       </c>
       <c r="E163" s="9" t="s">
         <v>159</v>
@@ -10910,11 +10910,11 @@
         <v>345</v>
       </c>
       <c r="B164" s="5">
-        <v>46109.579962187505</v>
+        <v>46109.74662885416</v>
       </c>
       <c r="C164" s="6"/>
       <c r="D164" s="5">
-        <v>46110.5883215625</v>
+        <v>46110.754988229164</v>
       </c>
       <c r="E164" s="6" t="s">
         <v>159</v>
@@ -10963,11 +10963,11 @@
         <v>346</v>
       </c>
       <c r="B165" s="8">
-        <v>46109.57997122685</v>
+        <v>46109.74663789352</v>
       </c>
       <c r="C165" s="9"/>
       <c r="D165" s="8">
-        <v>46110.58834326389</v>
+        <v>46110.75500993055</v>
       </c>
       <c r="E165" s="9" t="s">
         <v>159</v>
@@ -11016,11 +11016,11 @@
         <v>347</v>
       </c>
       <c r="B166" s="5">
-        <v>46109.579979409726</v>
+        <v>46109.74664607639</v>
       </c>
       <c r="C166" s="6"/>
       <c r="D166" s="5">
-        <v>46110.58836471065</v>
+        <v>46110.75503137731</v>
       </c>
       <c r="E166" s="6" t="s">
         <v>159</v>
@@ -11069,11 +11069,11 @@
         <v>348</v>
       </c>
       <c r="B167" s="8">
-        <v>46109.57998686343</v>
+        <v>46109.74665353009</v>
       </c>
       <c r="C167" s="9"/>
       <c r="D167" s="8">
-        <v>46110.588387951386</v>
+        <v>46110.75505461806</v>
       </c>
       <c r="E167" s="9" t="s">
         <v>159</v>
@@ -11122,11 +11122,11 @@
         <v>349</v>
       </c>
       <c r="B168" s="5">
-        <v>46109.57999479167</v>
+        <v>46109.74666145833</v>
       </c>
       <c r="C168" s="6"/>
       <c r="D168" s="5">
-        <v>46110.588415763894</v>
+        <v>46110.75508243055</v>
       </c>
       <c r="E168" s="6" t="s">
         <v>159</v>
@@ -11175,11 +11175,11 @@
         <v>350</v>
       </c>
       <c r="B169" s="8">
-        <v>46109.5800022801</v>
+        <v>46109.746668946755</v>
       </c>
       <c r="C169" s="9"/>
       <c r="D169" s="8">
-        <v>46110.58845435185</v>
+        <v>46110.75512101852</v>
       </c>
       <c r="E169" s="9" t="s">
         <v>159</v>
@@ -11228,11 +11228,11 @@
         <v>351</v>
       </c>
       <c r="B170" s="5">
-        <v>46073.41843864584</v>
+        <v>46073.5851053125</v>
       </c>
       <c r="C170" s="6"/>
       <c r="D170" s="5">
-        <v>46110.59601243056</v>
+        <v>46110.76267909722</v>
       </c>
       <c r="E170" s="6" t="s">
         <v>352</v>
@@ -11291,11 +11291,11 @@
         <v>353</v>
       </c>
       <c r="B171" s="8">
-        <v>46109.58042966435</v>
+        <v>46109.74709633102</v>
       </c>
       <c r="C171" s="9"/>
       <c r="D171" s="8">
-        <v>46110.59507837963</v>
+        <v>46110.7617450463</v>
       </c>
       <c r="E171" s="9" t="s">
         <v>159</v>
@@ -11344,11 +11344,11 @@
         <v>355</v>
       </c>
       <c r="B172" s="5">
-        <v>46109.58043918981</v>
+        <v>46109.747105856484</v>
       </c>
       <c r="C172" s="6"/>
       <c r="D172" s="5">
-        <v>46110.59511311342</v>
+        <v>46110.76177978009</v>
       </c>
       <c r="E172" s="6" t="s">
         <v>159</v>
@@ -11397,11 +11397,11 @@
         <v>356</v>
       </c>
       <c r="B173" s="8">
-        <v>46109.5804471875</v>
+        <v>46109.747113854166</v>
       </c>
       <c r="C173" s="9"/>
       <c r="D173" s="8">
-        <v>46110.595146493055</v>
+        <v>46110.76181315973</v>
       </c>
       <c r="E173" s="9" t="s">
         <v>159</v>
@@ -11450,11 +11450,11 @@
         <v>357</v>
       </c>
       <c r="B174" s="5">
-        <v>46109.58045424768</v>
+        <v>46109.747120914355</v>
       </c>
       <c r="C174" s="6"/>
       <c r="D174" s="5">
-        <v>46110.59516684028</v>
+        <v>46110.76183350694</v>
       </c>
       <c r="E174" s="6" t="s">
         <v>159</v>
@@ -11503,11 +11503,11 @@
         <v>358</v>
       </c>
       <c r="B175" s="8">
-        <v>46109.58046193287</v>
+        <v>46109.74712859954</v>
       </c>
       <c r="C175" s="9"/>
       <c r="D175" s="8">
-        <v>46110.59519228009</v>
+        <v>46110.76185894676</v>
       </c>
       <c r="E175" s="9" t="s">
         <v>159</v>
@@ -11556,11 +11556,11 @@
         <v>359</v>
       </c>
       <c r="B176" s="5">
-        <v>46109.58046921296</v>
+        <v>46109.74713587963</v>
       </c>
       <c r="C176" s="6"/>
       <c r="D176" s="5">
-        <v>46110.595220937495</v>
+        <v>46110.76188760417</v>
       </c>
       <c r="E176" s="6" t="s">
         <v>159</v>
@@ -11609,11 +11609,11 @@
         <v>360</v>
       </c>
       <c r="B177" s="8">
-        <v>46109.58047538194</v>
+        <v>46109.74714204861</v>
       </c>
       <c r="C177" s="9"/>
       <c r="D177" s="8">
-        <v>46110.59529321759</v>
+        <v>46110.76195988426</v>
       </c>
       <c r="E177" s="9" t="s">
         <v>159</v>
@@ -11662,11 +11662,11 @@
         <v>361</v>
       </c>
       <c r="B178" s="5">
-        <v>46109.58048226852</v>
+        <v>46109.74714893519</v>
       </c>
       <c r="C178" s="6"/>
       <c r="D178" s="5">
-        <v>46110.595319942135</v>
+        <v>46110.76198660879</v>
       </c>
       <c r="E178" s="6" t="s">
         <v>159</v>
@@ -11715,11 +11715,11 @@
         <v>362</v>
       </c>
       <c r="B179" s="8">
-        <v>46109.58048696759</v>
+        <v>46109.747153634264</v>
       </c>
       <c r="C179" s="9"/>
       <c r="D179" s="8">
-        <v>46110.59536020833</v>
+        <v>46110.762026875</v>
       </c>
       <c r="E179" s="9" t="s">
         <v>159</v>
@@ -11768,11 +11768,11 @@
         <v>363</v>
       </c>
       <c r="B180" s="5">
-        <v>46109.58049346065</v>
+        <v>46109.747160127314</v>
       </c>
       <c r="C180" s="6"/>
       <c r="D180" s="5">
-        <v>46110.595366608795</v>
+        <v>46110.76203327546</v>
       </c>
       <c r="E180" s="6" t="s">
         <v>159</v>
@@ -11821,11 +11821,11 @@
         <v>364</v>
       </c>
       <c r="B181" s="8">
-        <v>46109.58049908565</v>
+        <v>46109.74716575231</v>
       </c>
       <c r="C181" s="9"/>
       <c r="D181" s="8">
-        <v>46110.59540766204</v>
+        <v>46110.762074328704</v>
       </c>
       <c r="E181" s="9" t="s">
         <v>159</v>
@@ -11874,11 +11874,11 @@
         <v>365</v>
       </c>
       <c r="B182" s="5">
-        <v>46109.580505624996</v>
+        <v>46109.74717229167</v>
       </c>
       <c r="C182" s="6"/>
       <c r="D182" s="5">
-        <v>46110.59545199074</v>
+        <v>46110.76211865741</v>
       </c>
       <c r="E182" s="6" t="s">
         <v>159</v>
@@ -11927,11 +11927,11 @@
         <v>366</v>
       </c>
       <c r="B183" s="8">
-        <v>46073.41846560185</v>
+        <v>46073.58513226852</v>
       </c>
       <c r="C183" s="9"/>
       <c r="D183" s="8">
-        <v>46091.31073520833</v>
+        <v>46091.477401875</v>
       </c>
       <c r="E183" s="9" t="s">
         <v>367</v>
@@ -11974,11 +11974,11 @@
         <v>369</v>
       </c>
       <c r="B184" s="5">
-        <v>46073.41846693287</v>
+        <v>46073.58513359954</v>
       </c>
       <c r="C184" s="6"/>
       <c r="D184" s="5">
-        <v>46110.59665930556</v>
+        <v>46110.76332597222</v>
       </c>
       <c r="E184" s="6" t="s">
         <v>370</v>
@@ -12035,11 +12035,11 @@
         <v>373</v>
       </c>
       <c r="B185" s="8">
-        <v>46109.58062421296</v>
+        <v>46109.74729087963</v>
       </c>
       <c r="C185" s="9"/>
       <c r="D185" s="8">
-        <v>46110.59762936343</v>
+        <v>46110.76429603009</v>
       </c>
       <c r="E185" s="9" t="s">
         <v>159</v>
@@ -12086,11 +12086,11 @@
         <v>375</v>
       </c>
       <c r="B186" s="5">
-        <v>46109.58063166667</v>
+        <v>46109.74729833333</v>
       </c>
       <c r="C186" s="6"/>
       <c r="D186" s="5">
-        <v>46110.59765388889</v>
+        <v>46110.76432055555</v>
       </c>
       <c r="E186" s="6" t="s">
         <v>159</v>
@@ -12137,11 +12137,11 @@
         <v>376</v>
       </c>
       <c r="B187" s="8">
-        <v>46109.58063894676</v>
+        <v>46109.747305613426</v>
       </c>
       <c r="C187" s="9"/>
       <c r="D187" s="8">
-        <v>46110.59900986111</v>
+        <v>46110.76567652778</v>
       </c>
       <c r="E187" s="9" t="s">
         <v>159</v>
@@ -12188,11 +12188,11 @@
         <v>377</v>
       </c>
       <c r="B188" s="5">
-        <v>46109.5806465625</v>
+        <v>46109.74731322916</v>
       </c>
       <c r="C188" s="6"/>
       <c r="D188" s="5">
-        <v>46110.5977025</v>
+        <v>46110.76436916667</v>
       </c>
       <c r="E188" s="6" t="s">
         <v>159</v>
@@ -12239,11 +12239,11 @@
         <v>378</v>
       </c>
       <c r="B189" s="8">
-        <v>46109.58065307871</v>
+        <v>46109.747319745366</v>
       </c>
       <c r="C189" s="9"/>
       <c r="D189" s="8">
-        <v>46110.597734849536</v>
+        <v>46110.76440151621</v>
       </c>
       <c r="E189" s="9" t="s">
         <v>159</v>
@@ -12290,11 +12290,11 @@
         <v>379</v>
       </c>
       <c r="B190" s="5">
-        <v>46109.58065802083</v>
+        <v>46109.7473246875</v>
       </c>
       <c r="C190" s="6"/>
       <c r="D190" s="5">
-        <v>46110.597760625</v>
+        <v>46110.764427291666</v>
       </c>
       <c r="E190" s="6" t="s">
         <v>159</v>
@@ -12341,11 +12341,11 @@
         <v>380</v>
       </c>
       <c r="B191" s="8">
-        <v>46109.58066460648</v>
+        <v>46109.747331273145</v>
       </c>
       <c r="C191" s="9"/>
       <c r="D191" s="8">
-        <v>46110.59778597222</v>
+        <v>46110.76445263889</v>
       </c>
       <c r="E191" s="9" t="s">
         <v>159</v>
@@ -12392,11 +12392,11 @@
         <v>381</v>
       </c>
       <c r="B192" s="5">
-        <v>46109.58066965277</v>
+        <v>46109.747336319444</v>
       </c>
       <c r="C192" s="6"/>
       <c r="D192" s="5">
-        <v>46110.59781510416</v>
+        <v>46110.764481770835</v>
       </c>
       <c r="E192" s="6" t="s">
         <v>159</v>
@@ -12443,11 +12443,11 @@
         <v>382</v>
       </c>
       <c r="B193" s="8">
-        <v>46109.58067623843</v>
+        <v>46109.74734290509</v>
       </c>
       <c r="C193" s="9"/>
       <c r="D193" s="8">
-        <v>46110.59784150463</v>
+        <v>46110.7645081713</v>
       </c>
       <c r="E193" s="9" t="s">
         <v>159</v>
@@ -12494,11 +12494,11 @@
         <v>383</v>
       </c>
       <c r="B194" s="5">
-        <v>46109.58068126158</v>
+        <v>46109.74734792824</v>
       </c>
       <c r="C194" s="6"/>
       <c r="D194" s="5">
-        <v>46110.59786517361</v>
+        <v>46110.76453184028</v>
       </c>
       <c r="E194" s="6" t="s">
         <v>159</v>
@@ -12545,11 +12545,11 @@
         <v>384</v>
       </c>
       <c r="B195" s="8">
-        <v>46109.58068734954</v>
+        <v>46109.7473540162</v>
       </c>
       <c r="C195" s="9"/>
       <c r="D195" s="8">
-        <v>46110.597892881946</v>
+        <v>46110.76455954861</v>
       </c>
       <c r="E195" s="9" t="s">
         <v>159</v>
@@ -12596,11 +12596,11 @@
         <v>385</v>
       </c>
       <c r="B196" s="5">
-        <v>46109.580692083335</v>
+        <v>46109.74735875</v>
       </c>
       <c r="C196" s="6"/>
       <c r="D196" s="5">
-        <v>46110.59793396991</v>
+        <v>46110.764600636576</v>
       </c>
       <c r="E196" s="6" t="s">
         <v>159</v>
@@ -12647,11 +12647,11 @@
         <v>386</v>
       </c>
       <c r="B197" s="8">
-        <v>46073.41846728009</v>
+        <v>46073.58513394676</v>
       </c>
       <c r="C197" s="9"/>
       <c r="D197" s="8">
-        <v>46110.601870555554</v>
+        <v>46110.76853722222</v>
       </c>
       <c r="E197" s="9" t="s">
         <v>387</v>
@@ -12710,11 +12710,11 @@
         <v>388</v>
       </c>
       <c r="B198" s="5">
-        <v>46109.58081209491</v>
+        <v>46109.74747876158</v>
       </c>
       <c r="C198" s="6"/>
       <c r="D198" s="5">
-        <v>46110.60186040509</v>
+        <v>46110.76852707176</v>
       </c>
       <c r="E198" s="6" t="s">
         <v>159</v>
@@ -12763,11 +12763,11 @@
         <v>390</v>
       </c>
       <c r="B199" s="8">
-        <v>46109.580822696764</v>
+        <v>46109.74748936342</v>
       </c>
       <c r="C199" s="9"/>
       <c r="D199" s="8">
-        <v>46110.60111913194</v>
+        <v>46110.76778579861</v>
       </c>
       <c r="E199" s="9" t="s">
         <v>159</v>
@@ -12816,11 +12816,11 @@
         <v>391</v>
       </c>
       <c r="B200" s="5">
-        <v>46109.58083466435</v>
+        <v>46109.74750133102</v>
       </c>
       <c r="C200" s="6"/>
       <c r="D200" s="5">
-        <v>46110.60114414352</v>
+        <v>46110.76781081018</v>
       </c>
       <c r="E200" s="6" t="s">
         <v>159</v>
@@ -12869,11 +12869,11 @@
         <v>392</v>
       </c>
       <c r="B201" s="8">
-        <v>46109.58207618055</v>
+        <v>46109.74874284722</v>
       </c>
       <c r="C201" s="9"/>
       <c r="D201" s="8">
-        <v>46110.601165092594</v>
+        <v>46110.76783175926</v>
       </c>
       <c r="E201" s="9" t="s">
         <v>159</v>
@@ -12922,11 +12922,11 @@
         <v>393</v>
       </c>
       <c r="B202" s="5">
-        <v>46109.58210113426</v>
+        <v>46109.74876780093</v>
       </c>
       <c r="C202" s="6"/>
       <c r="D202" s="5">
-        <v>46110.60118945602</v>
+        <v>46110.767856122686</v>
       </c>
       <c r="E202" s="6" t="s">
         <v>159</v>
@@ -12975,11 +12975,11 @@
         <v>394</v>
       </c>
       <c r="B203" s="8">
-        <v>46109.58213796296</v>
+        <v>46109.748804629635</v>
       </c>
       <c r="C203" s="9"/>
       <c r="D203" s="8">
-        <v>46110.60121335648</v>
+        <v>46110.76788002315</v>
       </c>
       <c r="E203" s="9" t="s">
         <v>159</v>
@@ -13028,11 +13028,11 @@
         <v>395</v>
       </c>
       <c r="B204" s="5">
-        <v>46109.5821703588</v>
+        <v>46109.74883702546</v>
       </c>
       <c r="C204" s="6"/>
       <c r="D204" s="5">
-        <v>46110.60124059027</v>
+        <v>46110.767907256944</v>
       </c>
       <c r="E204" s="6" t="s">
         <v>159</v>
@@ -13081,11 +13081,11 @@
         <v>396</v>
       </c>
       <c r="B205" s="8">
-        <v>46109.58218469907</v>
+        <v>46109.748851365744</v>
       </c>
       <c r="C205" s="9"/>
       <c r="D205" s="8">
-        <v>46110.601263159726</v>
+        <v>46110.76792982639</v>
       </c>
       <c r="E205" s="9" t="s">
         <v>159</v>
@@ -13134,11 +13134,11 @@
         <v>397</v>
       </c>
       <c r="B206" s="5">
-        <v>46109.58220013889</v>
+        <v>46109.74886680556</v>
       </c>
       <c r="C206" s="6"/>
       <c r="D206" s="5">
-        <v>46110.60128555556</v>
+        <v>46110.76795222222</v>
       </c>
       <c r="E206" s="6" t="s">
         <v>159</v>
@@ -13187,11 +13187,11 @@
         <v>398</v>
       </c>
       <c r="B207" s="8">
-        <v>46109.58221796296</v>
+        <v>46109.74888462963</v>
       </c>
       <c r="C207" s="9"/>
       <c r="D207" s="8">
-        <v>46110.60248951388</v>
+        <v>46110.769156180555</v>
       </c>
       <c r="E207" s="9" t="s">
         <v>159</v>
@@ -13240,11 +13240,11 @@
         <v>399</v>
       </c>
       <c r="B208" s="5">
-        <v>46109.582234305555</v>
+        <v>46109.74890097222</v>
       </c>
       <c r="C208" s="6"/>
       <c r="D208" s="5">
-        <v>46110.60137396991</v>
+        <v>46110.76804063657</v>
       </c>
       <c r="E208" s="6" t="s">
         <v>159</v>
@@ -13293,11 +13293,11 @@
         <v>400</v>
       </c>
       <c r="B209" s="8">
-        <v>46109.582254340276</v>
+        <v>46109.74892100695</v>
       </c>
       <c r="C209" s="9"/>
       <c r="D209" s="8">
-        <v>46110.60141618055</v>
+        <v>46110.76808284722</v>
       </c>
       <c r="E209" s="9" t="s">
         <v>159</v>
@@ -13346,11 +13346,11 @@
         <v>401</v>
       </c>
       <c r="B210" s="5">
-        <v>46073.418467615746</v>
+        <v>46073.5851342824</v>
       </c>
       <c r="C210" s="6"/>
       <c r="D210" s="5">
-        <v>46110.60557288195</v>
+        <v>46110.77223954861</v>
       </c>
       <c r="E210" s="6" t="s">
         <v>402</v>
@@ -13409,11 +13409,11 @@
         <v>403</v>
       </c>
       <c r="B211" s="8">
-        <v>46109.58233839121</v>
+        <v>46109.74900505787</v>
       </c>
       <c r="C211" s="9"/>
       <c r="D211" s="8">
-        <v>46110.604106203704</v>
+        <v>46110.77077287037</v>
       </c>
       <c r="E211" s="9" t="s">
         <v>159</v>
@@ -13460,11 +13460,11 @@
         <v>405</v>
       </c>
       <c r="B212" s="5">
-        <v>46109.58236053241</v>
+        <v>46109.749027199075</v>
       </c>
       <c r="C212" s="6"/>
       <c r="D212" s="5">
-        <v>46110.604140138894</v>
+        <v>46110.77080680555</v>
       </c>
       <c r="E212" s="6" t="s">
         <v>159</v>
@@ -13511,11 +13511,11 @@
         <v>406</v>
       </c>
       <c r="B213" s="8">
-        <v>46109.582379432875</v>
+        <v>46109.74904609953</v>
       </c>
       <c r="C213" s="9"/>
       <c r="D213" s="8">
-        <v>46110.60418172454</v>
+        <v>46110.7708483912</v>
       </c>
       <c r="E213" s="9" t="s">
         <v>159</v>
@@ -13562,11 +13562,11 @@
         <v>407</v>
       </c>
       <c r="B214" s="5">
-        <v>46109.58239538195</v>
+        <v>46109.749062048606</v>
       </c>
       <c r="C214" s="6"/>
       <c r="D214" s="5">
-        <v>46110.60423924768</v>
+        <v>46110.77090591435</v>
       </c>
       <c r="E214" s="6" t="s">
         <v>159</v>
@@ -13613,11 +13613,11 @@
         <v>408</v>
       </c>
       <c r="B215" s="8">
-        <v>46109.582411400464</v>
+        <v>46109.74907806713</v>
       </c>
       <c r="C215" s="9"/>
       <c r="D215" s="8">
-        <v>46110.604266064816</v>
+        <v>46110.77093273148</v>
       </c>
       <c r="E215" s="9" t="s">
         <v>159</v>
@@ -13664,11 +13664,11 @@
         <v>409</v>
       </c>
       <c r="B216" s="5">
-        <v>46109.58242619213</v>
+        <v>46109.749092858794</v>
       </c>
       <c r="C216" s="6"/>
       <c r="D216" s="5">
-        <v>46110.60431461806</v>
+        <v>46110.77098128472</v>
       </c>
       <c r="E216" s="6" t="s">
         <v>159</v>
@@ -13715,11 +13715,11 @@
         <v>410</v>
       </c>
       <c r="B217" s="8">
-        <v>46109.58244542824</v>
+        <v>46109.74911209491</v>
       </c>
       <c r="C217" s="9"/>
       <c r="D217" s="8">
-        <v>46110.60439371528</v>
+        <v>46110.77106038194</v>
       </c>
       <c r="E217" s="9" t="s">
         <v>159</v>
@@ -13766,11 +13766,11 @@
         <v>411</v>
       </c>
       <c r="B218" s="5">
-        <v>46109.58246013889</v>
+        <v>46109.74912680556</v>
       </c>
       <c r="C218" s="6"/>
       <c r="D218" s="5">
-        <v>46110.60440503473</v>
+        <v>46110.77107170139</v>
       </c>
       <c r="E218" s="6" t="s">
         <v>159</v>
@@ -13817,11 +13817,11 @@
         <v>412</v>
       </c>
       <c r="B219" s="8">
-        <v>46109.582476261574</v>
+        <v>46109.74914292824</v>
       </c>
       <c r="C219" s="9"/>
       <c r="D219" s="8">
-        <v>46110.60443559028</v>
+        <v>46110.77110225694</v>
       </c>
       <c r="E219" s="9" t="s">
         <v>159</v>
@@ -13868,11 +13868,11 @@
         <v>413</v>
       </c>
       <c r="B220" s="5">
-        <v>46109.58249086805</v>
+        <v>46109.74915753472</v>
       </c>
       <c r="C220" s="6"/>
       <c r="D220" s="5">
-        <v>46110.60457376158</v>
+        <v>46110.771240428236</v>
       </c>
       <c r="E220" s="6" t="s">
         <v>159</v>
@@ -13919,11 +13919,11 @@
         <v>414</v>
       </c>
       <c r="B221" s="8">
-        <v>46109.58250725694</v>
+        <v>46109.749173923614</v>
       </c>
       <c r="C221" s="9"/>
       <c r="D221" s="8">
-        <v>46110.60460189814</v>
+        <v>46110.771268564815</v>
       </c>
       <c r="E221" s="9" t="s">
         <v>159</v>
@@ -13970,11 +13970,11 @@
         <v>415</v>
       </c>
       <c r="B222" s="5">
-        <v>46109.58254850694</v>
+        <v>46109.74921517361</v>
       </c>
       <c r="C222" s="6"/>
       <c r="D222" s="5">
-        <v>46110.60465226852</v>
+        <v>46110.771318935185</v>
       </c>
       <c r="E222" s="6" t="s">
         <v>159</v>
@@ -14021,11 +14021,11 @@
         <v>416</v>
       </c>
       <c r="B223" s="8">
-        <v>46073.41846792824</v>
+        <v>46073.585134594905</v>
       </c>
       <c r="C223" s="9"/>
       <c r="D223" s="8">
-        <v>46110.605572361106</v>
+        <v>46110.77223902778</v>
       </c>
       <c r="E223" s="9" t="s">
         <v>417</v>
@@ -14084,11 +14084,11 @@
         <v>419</v>
       </c>
       <c r="B224" s="5">
-        <v>46109.58260872685</v>
+        <v>46109.74927539352</v>
       </c>
       <c r="C224" s="6"/>
       <c r="D224" s="5">
-        <v>46111.36834144676</v>
+        <v>46111.535008113424</v>
       </c>
       <c r="E224" s="6" t="s">
         <v>159</v>
@@ -14135,11 +14135,11 @@
         <v>420</v>
       </c>
       <c r="B225" s="8">
-        <v>46109.58263106481</v>
+        <v>46109.74929773148</v>
       </c>
       <c r="C225" s="9"/>
       <c r="D225" s="8">
-        <v>46111.368373206016</v>
+        <v>46111.53503987269</v>
       </c>
       <c r="E225" s="9" t="s">
         <v>159</v>
@@ -14186,11 +14186,11 @@
         <v>421</v>
       </c>
       <c r="B226" s="5">
-        <v>46109.582642442125</v>
+        <v>46109.749309108796</v>
       </c>
       <c r="C226" s="6"/>
       <c r="D226" s="5">
-        <v>46111.368397708335</v>
+        <v>46111.535064375</v>
       </c>
       <c r="E226" s="6" t="s">
         <v>159</v>
@@ -14237,11 +14237,11 @@
         <v>422</v>
       </c>
       <c r="B227" s="8">
-        <v>46109.582661990746</v>
+        <v>46109.7493286574</v>
       </c>
       <c r="C227" s="9"/>
       <c r="D227" s="8">
-        <v>46111.36842489583</v>
+        <v>46111.5350915625</v>
       </c>
       <c r="E227" s="9" t="s">
         <v>159</v>
@@ -14288,11 +14288,11 @@
         <v>423</v>
       </c>
       <c r="B228" s="5">
-        <v>46109.58285320602</v>
+        <v>46109.74951987268</v>
       </c>
       <c r="C228" s="6"/>
       <c r="D228" s="5">
-        <v>46111.36845170139</v>
+        <v>46111.535118368054</v>
       </c>
       <c r="E228" s="6" t="s">
         <v>159</v>
@@ -14339,11 +14339,11 @@
         <v>424</v>
       </c>
       <c r="B229" s="8">
-        <v>46109.58287784722</v>
+        <v>46109.74954451389</v>
       </c>
       <c r="C229" s="9"/>
       <c r="D229" s="8">
-        <v>46111.368479930556</v>
+        <v>46111.53514659722</v>
       </c>
       <c r="E229" s="9" t="s">
         <v>159</v>
@@ -14390,11 +14390,11 @@
         <v>425</v>
       </c>
       <c r="B230" s="5">
-        <v>46109.58289719907</v>
+        <v>46109.74956386574</v>
       </c>
       <c r="C230" s="6"/>
       <c r="D230" s="5">
-        <v>46111.3685036574</v>
+        <v>46111.535170324074</v>
       </c>
       <c r="E230" s="6" t="s">
         <v>159</v>
@@ -14441,11 +14441,11 @@
         <v>426</v>
       </c>
       <c r="B231" s="8">
-        <v>46109.582914004626</v>
+        <v>46109.7495806713</v>
       </c>
       <c r="C231" s="9"/>
       <c r="D231" s="8">
-        <v>46111.368527708335</v>
+        <v>46111.535194375</v>
       </c>
       <c r="E231" s="9" t="s">
         <v>159</v>
@@ -14492,11 +14492,11 @@
         <v>427</v>
       </c>
       <c r="B232" s="5">
-        <v>46109.582931736106</v>
+        <v>46109.74959840278</v>
       </c>
       <c r="C232" s="6"/>
       <c r="D232" s="5">
-        <v>46111.36855143518</v>
+        <v>46111.53521810185</v>
       </c>
       <c r="E232" s="6" t="s">
         <v>159</v>
@@ -14543,11 +14543,11 @@
         <v>428</v>
       </c>
       <c r="B233" s="8">
-        <v>46109.58294940973</v>
+        <v>46109.749616076384</v>
       </c>
       <c r="C233" s="9"/>
       <c r="D233" s="8">
-        <v>46111.3685787963</v>
+        <v>46111.53524546296</v>
       </c>
       <c r="E233" s="9" t="s">
         <v>159</v>
@@ -14594,11 +14594,11 @@
         <v>429</v>
       </c>
       <c r="B234" s="5">
-        <v>46109.58296900463</v>
+        <v>46109.749635671295</v>
       </c>
       <c r="C234" s="6"/>
       <c r="D234" s="5">
-        <v>46111.36861532407</v>
+        <v>46111.53528199074</v>
       </c>
       <c r="E234" s="6" t="s">
         <v>159</v>
@@ -14645,11 +14645,11 @@
         <v>430</v>
       </c>
       <c r="B235" s="8">
-        <v>46109.72620990741</v>
+        <v>46109.89287657407</v>
       </c>
       <c r="C235" s="9"/>
       <c r="D235" s="8">
-        <v>46111.368706203706</v>
+        <v>46111.53537287037</v>
       </c>
       <c r="E235" s="9" t="s">
         <v>159</v>
@@ -14696,11 +14696,11 @@
         <v>431</v>
       </c>
       <c r="B236" s="5">
-        <v>46073.418468240736</v>
+        <v>46073.58513490741</v>
       </c>
       <c r="C236" s="6"/>
       <c r="D236" s="5">
-        <v>46091.310734375</v>
+        <v>46091.477401041666</v>
       </c>
       <c r="E236" s="6" t="s">
         <v>432</v>
@@ -14743,11 +14743,11 @@
         <v>434</v>
       </c>
       <c r="B237" s="8">
-        <v>46073.418468564814</v>
+        <v>46073.58513523148</v>
       </c>
       <c r="C237" s="9"/>
       <c r="D237" s="8">
-        <v>46091.321923344905</v>
+        <v>46091.48859001158</v>
       </c>
       <c r="E237" s="9" t="s">
         <v>435</v>
@@ -14806,11 +14806,11 @@
         <v>438</v>
       </c>
       <c r="B238" s="5">
-        <v>46073.41846888889</v>
+        <v>46073.58513555556</v>
       </c>
       <c r="C238" s="6"/>
       <c r="D238" s="5">
-        <v>46107.617363391204</v>
+        <v>46107.78403005787</v>
       </c>
       <c r="E238" s="6" t="s">
         <v>439</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-06-15 13:30 UTC
</commit_message>
<xml_diff>
--- a/data/50001309 - ZITRON COLOMBIA BUGA BUENAVENTURA.xlsx
+++ b/data/50001309 - ZITRON COLOMBIA BUGA BUENAVENTURA.xlsx
@@ -9834,7 +9834,7 @@
       </c>
       <c r="C144" s="6"/>
       <c r="D144" s="5">
-        <v>46110.752998819444</v>
+        <v>46188.167922962966</v>
       </c>
       <c r="E144" s="6" t="s">
         <v>316</v>
@@ -9897,7 +9897,7 @@
       </c>
       <c r="C145" s="9"/>
       <c r="D145" s="8">
-        <v>46110.75192106482</v>
+        <v>46188.16844658565</v>
       </c>
       <c r="E145" s="9" t="s">
         <v>159</v>
@@ -9950,7 +9950,7 @@
       </c>
       <c r="C146" s="6"/>
       <c r="D146" s="5">
-        <v>46110.75199584491</v>
+        <v>46188.16844814815</v>
       </c>
       <c r="E146" s="6" t="s">
         <v>159</v>
@@ -10003,7 +10003,7 @@
       </c>
       <c r="C147" s="9"/>
       <c r="D147" s="8">
-        <v>46110.752027083334</v>
+        <v>46188.168449467594</v>
       </c>
       <c r="E147" s="9" t="s">
         <v>159</v>
@@ -10056,7 +10056,7 @@
       </c>
       <c r="C148" s="6"/>
       <c r="D148" s="5">
-        <v>46110.752052627315</v>
+        <v>46188.16845092592</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>159</v>
@@ -10109,7 +10109,7 @@
       </c>
       <c r="C149" s="9"/>
       <c r="D149" s="8">
-        <v>46110.75208019676</v>
+        <v>46188.168452094906</v>
       </c>
       <c r="E149" s="9" t="s">
         <v>159</v>
@@ -10162,7 +10162,7 @@
       </c>
       <c r="C150" s="6"/>
       <c r="D150" s="5">
-        <v>46110.752111458336</v>
+        <v>46188.16845350694</v>
       </c>
       <c r="E150" s="6" t="s">
         <v>159</v>
@@ -10215,7 +10215,7 @@
       </c>
       <c r="C151" s="9"/>
       <c r="D151" s="8">
-        <v>46110.752136400464</v>
+        <v>46188.16845494213</v>
       </c>
       <c r="E151" s="9" t="s">
         <v>159</v>
@@ -10268,7 +10268,7 @@
       </c>
       <c r="C152" s="6"/>
       <c r="D152" s="5">
-        <v>46110.75215878472</v>
+        <v>46188.16845658565</v>
       </c>
       <c r="E152" s="6" t="s">
         <v>159</v>
@@ -10321,7 +10321,7 @@
       </c>
       <c r="C153" s="9"/>
       <c r="D153" s="8">
-        <v>46110.752180763884</v>
+        <v>46188.16845791666</v>
       </c>
       <c r="E153" s="9" t="s">
         <v>159</v>
@@ -10374,7 +10374,7 @@
       </c>
       <c r="C154" s="6"/>
       <c r="D154" s="5">
-        <v>46110.75220524306</v>
+        <v>46188.168459189816</v>
       </c>
       <c r="E154" s="6" t="s">
         <v>159</v>
@@ -10427,7 +10427,7 @@
       </c>
       <c r="C155" s="9"/>
       <c r="D155" s="8">
-        <v>46110.75223005787</v>
+        <v>46188.16846033565</v>
       </c>
       <c r="E155" s="9" t="s">
         <v>159</v>
@@ -10480,7 +10480,7 @@
       </c>
       <c r="C156" s="6"/>
       <c r="D156" s="5">
-        <v>46110.752270509256</v>
+        <v>46188.16846162037</v>
       </c>
       <c r="E156" s="6" t="s">
         <v>159</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-16 14:48 UTC
</commit_message>
<xml_diff>
--- a/data/50001309 - ZITRON COLOMBIA BUGA BUENAVENTURA.xlsx
+++ b/data/50001309 - ZITRON COLOMBIA BUGA BUENAVENTURA.xlsx
@@ -10533,7 +10533,7 @@
       </c>
       <c r="C157" s="9"/>
       <c r="D157" s="8">
-        <v>46110.75564038195</v>
+        <v>46189.16756869213</v>
       </c>
       <c r="E157" s="9" t="s">
         <v>336</v>
@@ -10596,7 +10596,7 @@
       </c>
       <c r="C158" s="6"/>
       <c r="D158" s="5">
-        <v>46110.75482741898</v>
+        <v>46189.16798542824</v>
       </c>
       <c r="E158" s="6" t="s">
         <v>159</v>
@@ -10649,7 +10649,7 @@
       </c>
       <c r="C159" s="9"/>
       <c r="D159" s="8">
-        <v>46110.75485027778</v>
+        <v>46189.1679869213</v>
       </c>
       <c r="E159" s="9" t="s">
         <v>159</v>
@@ -10702,7 +10702,7 @@
       </c>
       <c r="C160" s="6"/>
       <c r="D160" s="5">
-        <v>46110.754874502316</v>
+        <v>46189.16798825232</v>
       </c>
       <c r="E160" s="6" t="s">
         <v>159</v>
@@ -10755,7 +10755,7 @@
       </c>
       <c r="C161" s="9"/>
       <c r="D161" s="8">
-        <v>46110.754882106485</v>
+        <v>46189.16798960648</v>
       </c>
       <c r="E161" s="9" t="s">
         <v>159</v>
@@ -10808,7 +10808,7 @@
       </c>
       <c r="C162" s="6"/>
       <c r="D162" s="5">
-        <v>46110.75837865741</v>
+        <v>46189.16799120371</v>
       </c>
       <c r="E162" s="6" t="s">
         <v>159</v>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="C163" s="9"/>
       <c r="D163" s="8">
-        <v>46110.754965810185</v>
+        <v>46189.16799271991</v>
       </c>
       <c r="E163" s="9" t="s">
         <v>159</v>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="C164" s="6"/>
       <c r="D164" s="5">
-        <v>46110.754988229164</v>
+        <v>46189.167994421296</v>
       </c>
       <c r="E164" s="6" t="s">
         <v>159</v>
@@ -10967,7 +10967,7 @@
       </c>
       <c r="C165" s="9"/>
       <c r="D165" s="8">
-        <v>46110.75500993055</v>
+        <v>46189.1679960301</v>
       </c>
       <c r="E165" s="9" t="s">
         <v>159</v>
@@ -11020,7 +11020,7 @@
       </c>
       <c r="C166" s="6"/>
       <c r="D166" s="5">
-        <v>46110.75503137731</v>
+        <v>46189.16799758102</v>
       </c>
       <c r="E166" s="6" t="s">
         <v>159</v>
@@ -11073,7 +11073,7 @@
       </c>
       <c r="C167" s="9"/>
       <c r="D167" s="8">
-        <v>46110.75505461806</v>
+        <v>46189.167999074074</v>
       </c>
       <c r="E167" s="9" t="s">
         <v>159</v>
@@ -11126,7 +11126,7 @@
       </c>
       <c r="C168" s="6"/>
       <c r="D168" s="5">
-        <v>46110.75508243055</v>
+        <v>46189.16800063658</v>
       </c>
       <c r="E168" s="6" t="s">
         <v>159</v>
@@ -11179,7 +11179,7 @@
       </c>
       <c r="C169" s="9"/>
       <c r="D169" s="8">
-        <v>46110.75512101852</v>
+        <v>46189.16800194445</v>
       </c>
       <c r="E169" s="9" t="s">
         <v>159</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-17 04:22 UTC
</commit_message>
<xml_diff>
--- a/data/50001309 - ZITRON COLOMBIA BUGA BUENAVENTURA.xlsx
+++ b/data/50001309 - ZITRON COLOMBIA BUGA BUENAVENTURA.xlsx
@@ -4310,7 +4310,7 @@
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="5">
-        <v>46110.760131076386</v>
+        <v>46190.16767924769</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>154</v>
@@ -4373,7 +4373,7 @@
       </c>
       <c r="C43" s="9"/>
       <c r="D43" s="8">
-        <v>46110.75974422454</v>
+        <v>46190.16799011574</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>159</v>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="5">
-        <v>46110.75977424769</v>
+        <v>46190.16799153935</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>159</v>
@@ -4479,7 +4479,7 @@
       </c>
       <c r="C45" s="9"/>
       <c r="D45" s="8">
-        <v>46110.75979293982</v>
+        <v>46190.16799284722</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>159</v>
@@ -4532,7 +4532,7 @@
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="5">
-        <v>46110.75982019676</v>
+        <v>46190.167994143514</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>159</v>
@@ -4585,7 +4585,7 @@
       </c>
       <c r="C47" s="9"/>
       <c r="D47" s="8">
-        <v>46110.759835902776</v>
+        <v>46190.16799534722</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>159</v>
@@ -4638,7 +4638,7 @@
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="5">
-        <v>46110.75987070602</v>
+        <v>46190.16799662037</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>166</v>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="C49" s="9"/>
       <c r="D49" s="8">
-        <v>46110.7598769676</v>
+        <v>46190.16799802083</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>159</v>
@@ -4744,7 +4744,7 @@
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="5">
-        <v>46110.759901736106</v>
+        <v>46190.167999513884</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>159</v>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="C51" s="9"/>
       <c r="D51" s="8">
-        <v>46110.75992268519</v>
+        <v>46190.16800085648</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>159</v>
@@ -4850,7 +4850,7 @@
       </c>
       <c r="C52" s="6"/>
       <c r="D52" s="5">
-        <v>46110.75995075231</v>
+        <v>46190.16800236111</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>159</v>
@@ -4903,7 +4903,7 @@
       </c>
       <c r="C53" s="9"/>
       <c r="D53" s="8">
-        <v>46110.7599783912</v>
+        <v>46190.16800384259</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>159</v>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="C54" s="6"/>
       <c r="D54" s="5">
-        <v>46110.760016238426</v>
+        <v>46190.168005266205</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>159</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-06-18 13:50 UTC
</commit_message>
<xml_diff>
--- a/data/50001309 - ZITRON COLOMBIA BUGA BUENAVENTURA.xlsx
+++ b/data/50001309 - ZITRON COLOMBIA BUGA BUENAVENTURA.xlsx
@@ -11232,7 +11232,7 @@
       </c>
       <c r="C170" s="6"/>
       <c r="D170" s="5">
-        <v>46110.76267909722</v>
+        <v>46191.16762900463</v>
       </c>
       <c r="E170" s="6" t="s">
         <v>352</v>
@@ -11295,7 +11295,7 @@
       </c>
       <c r="C171" s="9"/>
       <c r="D171" s="8">
-        <v>46110.7617450463</v>
+        <v>46191.16805202546</v>
       </c>
       <c r="E171" s="9" t="s">
         <v>159</v>
@@ -11348,7 +11348,7 @@
       </c>
       <c r="C172" s="6"/>
       <c r="D172" s="5">
-        <v>46110.76177978009</v>
+        <v>46191.16805349537</v>
       </c>
       <c r="E172" s="6" t="s">
         <v>159</v>
@@ -11401,7 +11401,7 @@
       </c>
       <c r="C173" s="9"/>
       <c r="D173" s="8">
-        <v>46110.76181315973</v>
+        <v>46191.1680547338</v>
       </c>
       <c r="E173" s="9" t="s">
         <v>159</v>
@@ -11454,7 +11454,7 @@
       </c>
       <c r="C174" s="6"/>
       <c r="D174" s="5">
-        <v>46110.76183350694</v>
+        <v>46191.16805612268</v>
       </c>
       <c r="E174" s="6" t="s">
         <v>159</v>
@@ -11507,7 +11507,7 @@
       </c>
       <c r="C175" s="9"/>
       <c r="D175" s="8">
-        <v>46110.76185894676</v>
+        <v>46191.16805734954</v>
       </c>
       <c r="E175" s="9" t="s">
         <v>159</v>
@@ -11560,7 +11560,7 @@
       </c>
       <c r="C176" s="6"/>
       <c r="D176" s="5">
-        <v>46110.76188760417</v>
+        <v>46191.168058553245</v>
       </c>
       <c r="E176" s="6" t="s">
         <v>159</v>
@@ -11613,7 +11613,7 @@
       </c>
       <c r="C177" s="9"/>
       <c r="D177" s="8">
-        <v>46110.76195988426</v>
+        <v>46191.168059814816</v>
       </c>
       <c r="E177" s="9" t="s">
         <v>159</v>
@@ -11666,7 +11666,7 @@
       </c>
       <c r="C178" s="6"/>
       <c r="D178" s="5">
-        <v>46110.76198660879</v>
+        <v>46191.168061018514</v>
       </c>
       <c r="E178" s="6" t="s">
         <v>159</v>
@@ -11719,7 +11719,7 @@
       </c>
       <c r="C179" s="9"/>
       <c r="D179" s="8">
-        <v>46110.762026875</v>
+        <v>46191.16806226852</v>
       </c>
       <c r="E179" s="9" t="s">
         <v>159</v>
@@ -11772,7 +11772,7 @@
       </c>
       <c r="C180" s="6"/>
       <c r="D180" s="5">
-        <v>46110.76203327546</v>
+        <v>46191.16806351852</v>
       </c>
       <c r="E180" s="6" t="s">
         <v>159</v>
@@ -11825,7 +11825,7 @@
       </c>
       <c r="C181" s="9"/>
       <c r="D181" s="8">
-        <v>46110.762074328704</v>
+        <v>46191.16806474537</v>
       </c>
       <c r="E181" s="9" t="s">
         <v>159</v>
@@ -11878,7 +11878,7 @@
       </c>
       <c r="C182" s="6"/>
       <c r="D182" s="5">
-        <v>46110.76211865741</v>
+        <v>46191.16806616898</v>
       </c>
       <c r="E182" s="6" t="s">
         <v>159</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-19 12:39 UTC
</commit_message>
<xml_diff>
--- a/data/50001309 - ZITRON COLOMBIA BUGA BUENAVENTURA.xlsx
+++ b/data/50001309 - ZITRON COLOMBIA BUGA BUENAVENTURA.xlsx
@@ -11978,7 +11978,7 @@
       </c>
       <c r="C184" s="6"/>
       <c r="D184" s="5">
-        <v>46110.76332597222</v>
+        <v>46192.1679825</v>
       </c>
       <c r="E184" s="6" t="s">
         <v>370</v>
@@ -12039,7 +12039,7 @@
       </c>
       <c r="C185" s="9"/>
       <c r="D185" s="8">
-        <v>46110.76429603009</v>
+        <v>46192.16904489583</v>
       </c>
       <c r="E185" s="9" t="s">
         <v>159</v>
@@ -12090,7 +12090,7 @@
       </c>
       <c r="C186" s="6"/>
       <c r="D186" s="5">
-        <v>46110.76432055555</v>
+        <v>46192.16910128472</v>
       </c>
       <c r="E186" s="6" t="s">
         <v>159</v>
@@ -12141,7 +12141,7 @@
       </c>
       <c r="C187" s="9"/>
       <c r="D187" s="8">
-        <v>46110.76567652778</v>
+        <v>46192.16911097222</v>
       </c>
       <c r="E187" s="9" t="s">
         <v>159</v>
@@ -12192,7 +12192,7 @@
       </c>
       <c r="C188" s="6"/>
       <c r="D188" s="5">
-        <v>46110.76436916667</v>
+        <v>46192.169137951394</v>
       </c>
       <c r="E188" s="6" t="s">
         <v>159</v>
@@ -12243,7 +12243,7 @@
       </c>
       <c r="C189" s="9"/>
       <c r="D189" s="8">
-        <v>46110.76440151621</v>
+        <v>46192.16919045139</v>
       </c>
       <c r="E189" s="9" t="s">
         <v>159</v>
@@ -12294,7 +12294,7 @@
       </c>
       <c r="C190" s="6"/>
       <c r="D190" s="5">
-        <v>46110.764427291666</v>
+        <v>46192.16921581019</v>
       </c>
       <c r="E190" s="6" t="s">
         <v>159</v>
@@ -12345,7 +12345,7 @@
       </c>
       <c r="C191" s="9"/>
       <c r="D191" s="8">
-        <v>46110.76445263889</v>
+        <v>46192.16925050926</v>
       </c>
       <c r="E191" s="9" t="s">
         <v>159</v>
@@ -12396,7 +12396,7 @@
       </c>
       <c r="C192" s="6"/>
       <c r="D192" s="5">
-        <v>46110.764481770835</v>
+        <v>46192.16927513889</v>
       </c>
       <c r="E192" s="6" t="s">
         <v>159</v>
@@ -12447,7 +12447,7 @@
       </c>
       <c r="C193" s="9"/>
       <c r="D193" s="8">
-        <v>46110.7645081713</v>
+        <v>46192.1693571412</v>
       </c>
       <c r="E193" s="9" t="s">
         <v>159</v>
@@ -12498,7 +12498,7 @@
       </c>
       <c r="C194" s="6"/>
       <c r="D194" s="5">
-        <v>46110.76453184028</v>
+        <v>46192.16938392361</v>
       </c>
       <c r="E194" s="6" t="s">
         <v>159</v>
@@ -12549,7 +12549,7 @@
       </c>
       <c r="C195" s="9"/>
       <c r="D195" s="8">
-        <v>46110.76455954861</v>
+        <v>46192.170623831014</v>
       </c>
       <c r="E195" s="9" t="s">
         <v>159</v>
@@ -12600,7 +12600,7 @@
       </c>
       <c r="C196" s="6"/>
       <c r="D196" s="5">
-        <v>46110.764600636576</v>
+        <v>46192.17068005787</v>
       </c>
       <c r="E196" s="6" t="s">
         <v>159</v>

</xml_diff>